<commit_message>
Integra la ablación de la función de aptitud en toda la documentación
- Libro (59 págs): nuevo cierre de la sección 5.6 con la Figura 11 (curva
  aptitud vs m, sin restricciones de rango) y la Tabla 12 (óptimos de F_apt
  y Fo sobre los 20 pares), con actualización de las listas de figuras y
  tablas; el texto explica el piso m*=0,30 en las 50 corridas, el óptimo
  trivial r=1 de Fo sobre la propuesta y la coincidencia del máximo real de
  Fo con nuestro óptimo (m~0,07), reforzando H2.
- Informe de avances (28 págs): nueva sección 12 con la curva y la Tabla 9;
  conclusiones renumeradas a 13; próximos pasos incluyen el experimento M3FD.
- Excel (11 hojas): hoja nueva Ablacion_Fo con los barridos y la comparativa.
- Presentación (18 láminas): lámina nueva tras la de PSO con la curva y la
  lectura del experimento, con notas del orador para la pregunta del tribunal.
</commit_message>
<xml_diff>
--- a/docs/Avances_Tesis_Tablas.xlsx
+++ b/docs/Avances_Tesis_Tablas.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wilcoxon" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ranking_Global" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deteccion_LLVIP" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablacion_Fo" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -533,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -726,6 +727,18 @@
       <c r="B19" s="6" t="inlineStr">
         <is>
           <t>mAP de YOLOv8n reentrenado por método sobre LLVIP (evaluación orientada a tarea)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Ablacion_Fo</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Ablación de la función de aptitud: barridos con la Fo del libro FPUNA y comparación de óptimos</t>
         </is>
       </c>
     </row>
@@ -966,6 +979,190 @@
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Lectura: toda fusión supera al visible solo (+0,12 a +0,14 en mAP@0,5); el infrarrojo solo es la modalidad más fuerte (0,957) y ninguna fusión lo supera (peatón nocturno = térmico); entre las fusiones, en banda estrecha (0,926–0,949), la propuesta es competitiva (0,936) sin ser líder. La superioridad en calidad de imagen no se traslada automáticamente a la detección (H3 parcial).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ablación de la función de aptitud (pedido de la revisión de avances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>El barrido 5×5 se repitió con la Fo del libro FPUNA (SSIM_avg + E_n + PSNR_n) y su rango m ∈ [0,3; 2,0], sobre la propuesta y sobre el operador clásico. En negrita el mejor por columna.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Resultado de los barridos con Fo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>En las 50 corridas (25 configuraciones × 2 operadores) el óptimo fue m* = 0,30, el piso del rango: los términos de fidelidad de Fo dominan a la entropía. Sobre la propuesta Fo eligió además r* = 1 (óptimo trivial); sobre el clásico, r* = 25.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Curva aptitud vs m (r = 25, sin restricciones): las tres curvas decrecen monótonamente en [0,5; 2,0] — ningún (n, T) puede converger allí — y el máximo real de Fo sobre la propuesta está en m ≈ 0,07, coincidente con el óptimo de F_apt (0,0703). Ver docs/figures/fig_aptitud_vs_m.png.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Variante (operador + aptitud)</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Qabf ↑</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Nabf ↓</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>SSIM ↑</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>SCD ↑</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>VIF ↑</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Propuesta + F_apt (r=25; m=0,070)</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>0.368</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Top-Hat clásico + Fo (r=25; m=0,30)</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="n">
+        <v>0.534</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>0.745</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>1.504</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>0.395</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Propuesta + Fo (r=1; m=0,30)</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>1.353</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>0.322</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Top-Hat clásico manual (r=5; m=1)</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>0.305</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>0.585</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>0.578</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>0.334</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Lectura: la propuesta con F_apt conserva el mejor perfil de limpieza y estructura (Nabf, SSIM); el óptimo de Fo sobre el clásico es competitivo en bordes y correlación al costo de 4,5× más artefactos; el de Fo sobre la propuesta confirma el óptimo trivial. La aptitud define el perfil del resultado (refuerza H2). Fuente: metrics_reports/fo_ablacion_comparativa.csv y pso_grid_search_fo_*.csv.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Integra los resultados M3FD en libro, avances, Excel, presentación y README
- Libro (61 págs): sección 5.5 retitulada (LLVIP y M3FD) y cerrada con el
  bloque de clases complementarias (Tabla 13); sexto hallazgo en 5.7,
  conclusión ampliada, RESUMEN/SUMMARY actualizados y referencia Liu et al.
  (2022). Se normalizan las negritas de las Tablas 12 y 13.
- Avances (29 págs): sección 13 con Tabla 10 y lectura; conclusiones a 14.
- Excel (12 hojas): hoja nueva Deteccion_M3FD (0 errores de fórmula).
- Presentación (19 láminas): lámina de clases complementarias con barras
  agrupadas People/Lamp; agenda actualizada.
- README: resultados del experimento en la sección 8.1.
</commit_message>
<xml_diff>
--- a/docs/Avances_Tesis_Tablas.xlsx
+++ b/docs/Avances_Tesis_Tablas.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ranking_Global" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deteccion_LLVIP" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablacion_Fo" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deteccion_M3FD" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -534,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -739,6 +740,18 @@
       <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Ablación de la función de aptitud: barridos con la Fo del libro FPUNA y comparación de óptimos</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Deteccion_M3FD</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Clases complementarias en M3FD: AP por clase con un detector único VIS+IR (People/IR, Lamp/VIS)</t>
         </is>
       </c>
     </row>
@@ -1163,6 +1176,284 @@
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Lectura: la propuesta con F_apt conserva el mejor perfil de limpieza y estructura (Nabf, SSIM); el óptimo de Fo sobre el clásico es competitivo en bordes y correlación al costo de 4,5× más artefactos; el de Fo sobre la propuesta confirma el óptimo trivial. La aptitud define el perfil del resultado (refuerza H2). Fuente: metrics_reports/fo_ablacion_comparativa.csv y pso_grid_search_fo_*.csv.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clases complementarias en M3FD — un detector único VIS+IR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>YOLOv8n entrenado con las imágenes de ambas modalidades mezcladas (4.000 imágenes, 40 épocas) y evaluado por inferencia sobre cada entrada. People domina en IR (térmica); Lamp solo se ve en VIS. En negrita el mejor por columna.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Entrada del detector</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>AP@0,5 People ↑</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>AP@0,5 Lamp ↑</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Promedio del par ↑</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>mAP@0,5 (6 clases) ↑</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>VIS (solo)</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>0.157</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>0.245</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>IR (solo)</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>0.191</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Pirámide de Laplace (LP)</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>0.215</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Ratio Pyramid (RP)</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>0.231</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Wavelet discreta (DWT)</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>0.228</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Dual-Tree Complex Wavelet (DTCWT)</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>0.229</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Curvelet (CVT)</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>0.228</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Top-Hat clásico (r=5; m=1)</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>0.198</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>PSO FPUNA (clásico + Fo; r=25; m=0,30)</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>0.174</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>0.229</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Propuesta + Fo (r=1; m=0,30)</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>0.238</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Propuesta + F_apt (r=25; m=0,070)</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>0.239</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Lectura: complementariedad extrema (IR ciego a Lamp: 0,018; VIS débil en People). Las mejores fusiones superan en el promedio del par a ambas modalidades individuales (RP 0,165 y propuesta 0,162 vs VIS 0,157 e IR 0,119): detectan ambas clases en una sola imagen. La propuesta es la mejor fusión en mAP global (0,239) y en People (0,207), y F_apt supera a Fo en las dos clases clave. Fuente: metrics_reports/detection_m3fd_map.csv.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Avances, Excel y deck: completa el paralelo F_o vs F_apt en detección
- Avances (31 págs): fila Propuesta_Fo en la tabla LLVIP y en la gráfica de
  barras; línea del Wilcoxon (8/12 a favor de F_apt) en la ablación; nueva
  página 12 (continuación) con la comparación cualitativa de aptitudes.
- Excel: hoja Deteccion_LLVIP con ambas configs (F_apt y Fo); 0 errores.
- Deck (20 láminas): barras de LLVIP con las dos configs de la propuesta
  (F_apt granate, Fo rosa); lámina de ablación con el Wilcoxon 8/12.
</commit_message>
<xml_diff>
--- a/docs/Avances_Tesis_Tablas.xlsx
+++ b/docs/Avances_Tesis_Tablas.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -972,7 +972,7 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>PROPUESTA NOVEDOSA (r=25, m=0,070)</t>
+          <t>Propuesta · F_apt (r=25, m=0,070)</t>
         </is>
       </c>
       <c r="B13" s="18" t="n">
@@ -988,8 +988,27 @@
         <v>0.8585</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Propuesta · Fo (r=1, m=0,30)</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="n">
+        <v>0.9221</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>0.6188</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>0.9344</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>0.8014</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Lectura: toda fusión supera al visible solo (+0,12 a +0,14 en mAP@0,5); el infrarrojo solo es la modalidad más fuerte (0,957) y ninguna fusión lo supera (peatón nocturno = térmico); entre las fusiones, en banda estrecha (0,926–0,949), la propuesta es competitiva (0,936) sin ser líder. La superioridad en calidad de imagen no se traslada automáticamente a la detección (H3 parcial).</t>
         </is>

</xml_diff>

<commit_message>
Anexos: peso m con cuatro decimales
La columna m pasa de tres a cuatro decimales en los anexos del informe y en la hoja
PSO_por_Escena. Gana precision en las 16 filas (de 500) que no alcanzaron el limite del
rango: 0,910 -> 0,9104, 1,363 -> 1,3634, etc. Las 484 filas restantes se leen 0,3000
porque el valor es exactamente el limite inferior del intervalo publicado, donde el PSO
recorta las posiciones.
</commit_message>
<xml_diff>
--- a/docs/Avances_Tesis_Tablas.xlsx
+++ b/docs/Avances_Tesis_Tablas.xlsx
@@ -8117,7 +8117,7 @@
       <c r="D5" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F5" s="20" t="n">
@@ -8150,7 +8150,7 @@
       <c r="D6" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F6" s="20" t="n">
@@ -8183,7 +8183,7 @@
       <c r="D7" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="12" t="n">
         <v>0.9104</v>
       </c>
       <c r="F7" s="20" t="n">
@@ -8216,7 +8216,7 @@
       <c r="D8" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F8" s="20" t="n">
@@ -8249,7 +8249,7 @@
       <c r="D9" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F9" s="21" t="n">
@@ -8282,7 +8282,7 @@
       <c r="D10" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F10" s="20" t="n">
@@ -8315,7 +8315,7 @@
       <c r="D11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F11" s="20" t="n">
@@ -8348,7 +8348,7 @@
       <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F12" s="20" t="n">
@@ -8381,7 +8381,7 @@
       <c r="D13" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E13" s="16" t="n">
+      <c r="E13" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F13" s="20" t="n">
@@ -8414,7 +8414,7 @@
       <c r="D14" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E14" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F14" s="20" t="n">
@@ -8447,7 +8447,7 @@
       <c r="D15" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="16" t="n">
+      <c r="E15" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F15" s="20" t="n">
@@ -8480,7 +8480,7 @@
       <c r="D16" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E16" s="16" t="n">
+      <c r="E16" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F16" s="20" t="n">
@@ -8513,7 +8513,7 @@
       <c r="D17" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="16" t="n">
+      <c r="E17" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F17" s="20" t="n">
@@ -8546,7 +8546,7 @@
       <c r="D18" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="16" t="n">
+      <c r="E18" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F18" s="20" t="n">
@@ -8579,7 +8579,7 @@
       <c r="D19" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="16" t="n">
+      <c r="E19" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F19" s="20" t="n">
@@ -8612,7 +8612,7 @@
       <c r="D20" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="16" t="n">
+      <c r="E20" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F20" s="20" t="n">
@@ -8645,7 +8645,7 @@
       <c r="D21" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="16" t="n">
+      <c r="E21" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F21" s="20" t="n">
@@ -8678,7 +8678,7 @@
       <c r="D22" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="16" t="n">
+      <c r="E22" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F22" s="20" t="n">
@@ -8711,7 +8711,7 @@
       <c r="D23" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E23" s="16" t="n">
+      <c r="E23" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F23" s="20" t="n">
@@ -8744,7 +8744,7 @@
       <c r="D24" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="16" t="n">
+      <c r="E24" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F24" s="20" t="n">
@@ -8777,7 +8777,7 @@
       <c r="D25" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E25" s="16" t="n">
+      <c r="E25" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F25" s="20" t="n">
@@ -8810,7 +8810,7 @@
       <c r="D26" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E26" s="16" t="n">
+      <c r="E26" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F26" s="20" t="n">
@@ -8843,7 +8843,7 @@
       <c r="D27" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E27" s="16" t="n">
+      <c r="E27" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F27" s="20" t="n">
@@ -8876,7 +8876,7 @@
       <c r="D28" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="16" t="n">
+      <c r="E28" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F28" s="20" t="n">
@@ -8909,7 +8909,7 @@
       <c r="D29" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E29" s="16" t="n">
+      <c r="E29" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F29" s="20" t="n">
@@ -8946,7 +8946,7 @@
       <c r="D30" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="17" t="n">
+      <c r="E30" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F30" s="21" t="n">
@@ -8979,7 +8979,7 @@
       <c r="D31" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="16" t="n">
+      <c r="E31" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F31" s="20" t="n">
@@ -9012,7 +9012,7 @@
       <c r="D32" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E32" s="16" t="n">
+      <c r="E32" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F32" s="20" t="n">
@@ -9045,7 +9045,7 @@
       <c r="D33" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E33" s="16" t="n">
+      <c r="E33" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F33" s="20" t="n">
@@ -9078,7 +9078,7 @@
       <c r="D34" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E34" s="16" t="n">
+      <c r="E34" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F34" s="20" t="n">
@@ -9111,7 +9111,7 @@
       <c r="D35" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E35" s="16" t="n">
+      <c r="E35" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F35" s="20" t="n">
@@ -9144,7 +9144,7 @@
       <c r="D36" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E36" s="16" t="n">
+      <c r="E36" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F36" s="20" t="n">
@@ -9177,7 +9177,7 @@
       <c r="D37" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E37" s="16" t="n">
+      <c r="E37" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F37" s="20" t="n">
@@ -9210,7 +9210,7 @@
       <c r="D38" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E38" s="16" t="n">
+      <c r="E38" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F38" s="20" t="n">
@@ -9243,7 +9243,7 @@
       <c r="D39" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E39" s="16" t="n">
+      <c r="E39" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F39" s="20" t="n">
@@ -9276,7 +9276,7 @@
       <c r="D40" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E40" s="16" t="n">
+      <c r="E40" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F40" s="20" t="n">
@@ -9309,7 +9309,7 @@
       <c r="D41" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E41" s="16" t="n">
+      <c r="E41" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F41" s="20" t="n">
@@ -9342,7 +9342,7 @@
       <c r="D42" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E42" s="16" t="n">
+      <c r="E42" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F42" s="20" t="n">
@@ -9375,7 +9375,7 @@
       <c r="D43" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E43" s="16" t="n">
+      <c r="E43" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F43" s="20" t="n">
@@ -9408,7 +9408,7 @@
       <c r="D44" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E44" s="16" t="n">
+      <c r="E44" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F44" s="20" t="n">
@@ -9441,7 +9441,7 @@
       <c r="D45" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E45" s="16" t="n">
+      <c r="E45" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F45" s="20" t="n">
@@ -9474,7 +9474,7 @@
       <c r="D46" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E46" s="16" t="n">
+      <c r="E46" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F46" s="20" t="n">
@@ -9507,7 +9507,7 @@
       <c r="D47" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E47" s="16" t="n">
+      <c r="E47" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F47" s="20" t="n">
@@ -9540,7 +9540,7 @@
       <c r="D48" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E48" s="16" t="n">
+      <c r="E48" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F48" s="20" t="n">
@@ -9573,7 +9573,7 @@
       <c r="D49" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E49" s="16" t="n">
+      <c r="E49" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F49" s="20" t="n">
@@ -9606,7 +9606,7 @@
       <c r="D50" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E50" s="16" t="n">
+      <c r="E50" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F50" s="20" t="n">
@@ -9639,7 +9639,7 @@
       <c r="D51" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E51" s="16" t="n">
+      <c r="E51" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F51" s="20" t="n">
@@ -9672,7 +9672,7 @@
       <c r="D52" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E52" s="16" t="n">
+      <c r="E52" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F52" s="20" t="n">
@@ -9705,7 +9705,7 @@
       <c r="D53" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E53" s="16" t="n">
+      <c r="E53" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F53" s="20" t="n">
@@ -9738,7 +9738,7 @@
       <c r="D54" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E54" s="16" t="n">
+      <c r="E54" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F54" s="20" t="n">
@@ -9775,7 +9775,7 @@
       <c r="D55" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E55" s="16" t="n">
+      <c r="E55" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F55" s="20" t="n">
@@ -9808,7 +9808,7 @@
       <c r="D56" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E56" s="17" t="n">
+      <c r="E56" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F56" s="21" t="n">
@@ -9841,7 +9841,7 @@
       <c r="D57" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E57" s="16" t="n">
+      <c r="E57" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F57" s="20" t="n">
@@ -9874,7 +9874,7 @@
       <c r="D58" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="E58" s="16" t="n">
+      <c r="E58" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F58" s="20" t="n">
@@ -9907,7 +9907,7 @@
       <c r="D59" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E59" s="16" t="n">
+      <c r="E59" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F59" s="20" t="n">
@@ -9940,7 +9940,7 @@
       <c r="D60" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E60" s="16" t="n">
+      <c r="E60" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F60" s="20" t="n">
@@ -9973,7 +9973,7 @@
       <c r="D61" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E61" s="16" t="n">
+      <c r="E61" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F61" s="20" t="n">
@@ -10006,7 +10006,7 @@
       <c r="D62" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E62" s="16" t="n">
+      <c r="E62" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F62" s="20" t="n">
@@ -10039,7 +10039,7 @@
       <c r="D63" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E63" s="16" t="n">
+      <c r="E63" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F63" s="20" t="n">
@@ -10072,7 +10072,7 @@
       <c r="D64" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E64" s="16" t="n">
+      <c r="E64" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F64" s="20" t="n">
@@ -10105,7 +10105,7 @@
       <c r="D65" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E65" s="16" t="n">
+      <c r="E65" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F65" s="20" t="n">
@@ -10138,7 +10138,7 @@
       <c r="D66" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E66" s="16" t="n">
+      <c r="E66" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F66" s="20" t="n">
@@ -10171,7 +10171,7 @@
       <c r="D67" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E67" s="16" t="n">
+      <c r="E67" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F67" s="20" t="n">
@@ -10204,7 +10204,7 @@
       <c r="D68" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E68" s="16" t="n">
+      <c r="E68" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F68" s="20" t="n">
@@ -10237,7 +10237,7 @@
       <c r="D69" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E69" s="16" t="n">
+      <c r="E69" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F69" s="20" t="n">
@@ -10270,7 +10270,7 @@
       <c r="D70" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E70" s="16" t="n">
+      <c r="E70" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F70" s="20" t="n">
@@ -10303,7 +10303,7 @@
       <c r="D71" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E71" s="16" t="n">
+      <c r="E71" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F71" s="20" t="n">
@@ -10336,7 +10336,7 @@
       <c r="D72" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E72" s="16" t="n">
+      <c r="E72" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F72" s="20" t="n">
@@ -10369,7 +10369,7 @@
       <c r="D73" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E73" s="16" t="n">
+      <c r="E73" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F73" s="20" t="n">
@@ -10402,7 +10402,7 @@
       <c r="D74" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E74" s="16" t="n">
+      <c r="E74" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F74" s="20" t="n">
@@ -10435,7 +10435,7 @@
       <c r="D75" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E75" s="16" t="n">
+      <c r="E75" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F75" s="20" t="n">
@@ -10468,7 +10468,7 @@
       <c r="D76" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E76" s="16" t="n">
+      <c r="E76" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F76" s="20" t="n">
@@ -10501,7 +10501,7 @@
       <c r="D77" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E77" s="16" t="n">
+      <c r="E77" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F77" s="20" t="n">
@@ -10534,7 +10534,7 @@
       <c r="D78" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E78" s="16" t="n">
+      <c r="E78" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F78" s="20" t="n">
@@ -10567,7 +10567,7 @@
       <c r="D79" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E79" s="16" t="n">
+      <c r="E79" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F79" s="20" t="n">
@@ -10604,7 +10604,7 @@
       <c r="D80" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E80" s="16" t="n">
+      <c r="E80" s="12" t="n">
         <v>1.5353</v>
       </c>
       <c r="F80" s="20" t="n">
@@ -10637,7 +10637,7 @@
       <c r="D81" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="E81" s="17" t="n">
+      <c r="E81" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F81" s="21" t="n">
@@ -10670,7 +10670,7 @@
       <c r="D82" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E82" s="16" t="n">
+      <c r="E82" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F82" s="20" t="n">
@@ -10703,7 +10703,7 @@
       <c r="D83" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E83" s="16" t="n">
+      <c r="E83" s="12" t="n">
         <v>1.3634</v>
       </c>
       <c r="F83" s="20" t="n">
@@ -10736,7 +10736,7 @@
       <c r="D84" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="E84" s="16" t="n">
+      <c r="E84" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F84" s="20" t="n">
@@ -10769,7 +10769,7 @@
       <c r="D85" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E85" s="16" t="n">
+      <c r="E85" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F85" s="20" t="n">
@@ -10802,7 +10802,7 @@
       <c r="D86" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E86" s="16" t="n">
+      <c r="E86" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F86" s="20" t="n">
@@ -10835,7 +10835,7 @@
       <c r="D87" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E87" s="16" t="n">
+      <c r="E87" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F87" s="20" t="n">
@@ -10868,7 +10868,7 @@
       <c r="D88" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E88" s="16" t="n">
+      <c r="E88" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F88" s="20" t="n">
@@ -10901,7 +10901,7 @@
       <c r="D89" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E89" s="16" t="n">
+      <c r="E89" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F89" s="20" t="n">
@@ -10934,7 +10934,7 @@
       <c r="D90" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E90" s="16" t="n">
+      <c r="E90" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F90" s="20" t="n">
@@ -10967,7 +10967,7 @@
       <c r="D91" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E91" s="16" t="n">
+      <c r="E91" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F91" s="20" t="n">
@@ -11000,7 +11000,7 @@
       <c r="D92" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E92" s="16" t="n">
+      <c r="E92" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F92" s="20" t="n">
@@ -11033,7 +11033,7 @@
       <c r="D93" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E93" s="16" t="n">
+      <c r="E93" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F93" s="20" t="n">
@@ -11066,7 +11066,7 @@
       <c r="D94" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E94" s="16" t="n">
+      <c r="E94" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F94" s="20" t="n">
@@ -11099,7 +11099,7 @@
       <c r="D95" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E95" s="16" t="n">
+      <c r="E95" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F95" s="20" t="n">
@@ -11132,7 +11132,7 @@
       <c r="D96" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E96" s="16" t="n">
+      <c r="E96" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F96" s="20" t="n">
@@ -11165,7 +11165,7 @@
       <c r="D97" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E97" s="16" t="n">
+      <c r="E97" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F97" s="20" t="n">
@@ -11198,7 +11198,7 @@
       <c r="D98" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E98" s="16" t="n">
+      <c r="E98" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F98" s="20" t="n">
@@ -11231,7 +11231,7 @@
       <c r="D99" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E99" s="16" t="n">
+      <c r="E99" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F99" s="20" t="n">
@@ -11264,7 +11264,7 @@
       <c r="D100" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E100" s="16" t="n">
+      <c r="E100" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F100" s="20" t="n">
@@ -11297,7 +11297,7 @@
       <c r="D101" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E101" s="16" t="n">
+      <c r="E101" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F101" s="20" t="n">
@@ -11330,7 +11330,7 @@
       <c r="D102" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E102" s="16" t="n">
+      <c r="E102" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F102" s="20" t="n">
@@ -11363,7 +11363,7 @@
       <c r="D103" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E103" s="16" t="n">
+      <c r="E103" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F103" s="20" t="n">
@@ -11396,7 +11396,7 @@
       <c r="D104" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E104" s="16" t="n">
+      <c r="E104" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F104" s="20" t="n">
@@ -11433,7 +11433,7 @@
       <c r="D105" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E105" s="16" t="n">
+      <c r="E105" s="12" t="n">
         <v>0.9476</v>
       </c>
       <c r="F105" s="20" t="n">
@@ -11466,7 +11466,7 @@
       <c r="D106" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E106" s="17" t="n">
+      <c r="E106" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F106" s="21" t="n">
@@ -11499,7 +11499,7 @@
       <c r="D107" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E107" s="16" t="n">
+      <c r="E107" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F107" s="20" t="n">
@@ -11532,7 +11532,7 @@
       <c r="D108" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E108" s="16" t="n">
+      <c r="E108" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F108" s="20" t="n">
@@ -11565,7 +11565,7 @@
       <c r="D109" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E109" s="16" t="n">
+      <c r="E109" s="12" t="n">
         <v>0.4554</v>
       </c>
       <c r="F109" s="20" t="n">
@@ -11598,7 +11598,7 @@
       <c r="D110" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E110" s="16" t="n">
+      <c r="E110" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F110" s="20" t="n">
@@ -11631,7 +11631,7 @@
       <c r="D111" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E111" s="16" t="n">
+      <c r="E111" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F111" s="20" t="n">
@@ -11664,7 +11664,7 @@
       <c r="D112" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E112" s="16" t="n">
+      <c r="E112" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F112" s="20" t="n">
@@ -11697,7 +11697,7 @@
       <c r="D113" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E113" s="16" t="n">
+      <c r="E113" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F113" s="20" t="n">
@@ -11730,7 +11730,7 @@
       <c r="D114" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E114" s="16" t="n">
+      <c r="E114" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F114" s="20" t="n">
@@ -11763,7 +11763,7 @@
       <c r="D115" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E115" s="16" t="n">
+      <c r="E115" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F115" s="20" t="n">
@@ -11796,7 +11796,7 @@
       <c r="D116" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E116" s="16" t="n">
+      <c r="E116" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F116" s="20" t="n">
@@ -11829,7 +11829,7 @@
       <c r="D117" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E117" s="16" t="n">
+      <c r="E117" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F117" s="20" t="n">
@@ -11862,7 +11862,7 @@
       <c r="D118" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E118" s="16" t="n">
+      <c r="E118" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F118" s="20" t="n">
@@ -11895,7 +11895,7 @@
       <c r="D119" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E119" s="16" t="n">
+      <c r="E119" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F119" s="20" t="n">
@@ -11928,7 +11928,7 @@
       <c r="D120" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="E120" s="16" t="n">
+      <c r="E120" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F120" s="20" t="n">
@@ -11961,7 +11961,7 @@
       <c r="D121" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E121" s="16" t="n">
+      <c r="E121" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F121" s="20" t="n">
@@ -11994,7 +11994,7 @@
       <c r="D122" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E122" s="16" t="n">
+      <c r="E122" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F122" s="20" t="n">
@@ -12027,7 +12027,7 @@
       <c r="D123" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E123" s="16" t="n">
+      <c r="E123" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F123" s="20" t="n">
@@ -12060,7 +12060,7 @@
       <c r="D124" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E124" s="16" t="n">
+      <c r="E124" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F124" s="20" t="n">
@@ -12093,7 +12093,7 @@
       <c r="D125" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E125" s="16" t="n">
+      <c r="E125" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F125" s="20" t="n">
@@ -12126,7 +12126,7 @@
       <c r="D126" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E126" s="16" t="n">
+      <c r="E126" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F126" s="20" t="n">
@@ -12159,7 +12159,7 @@
       <c r="D127" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E127" s="16" t="n">
+      <c r="E127" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F127" s="20" t="n">
@@ -12192,7 +12192,7 @@
       <c r="D128" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E128" s="16" t="n">
+      <c r="E128" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F128" s="20" t="n">
@@ -12225,7 +12225,7 @@
       <c r="D129" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E129" s="16" t="n">
+      <c r="E129" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F129" s="20" t="n">
@@ -12262,7 +12262,7 @@
       <c r="D130" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E130" s="17" t="n">
+      <c r="E130" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F130" s="21" t="n">
@@ -12295,7 +12295,7 @@
       <c r="D131" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="E131" s="16" t="n">
+      <c r="E131" s="12" t="n">
         <v>0.3775</v>
       </c>
       <c r="F131" s="20" t="n">
@@ -12328,7 +12328,7 @@
       <c r="D132" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="E132" s="16" t="n">
+      <c r="E132" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F132" s="20" t="n">
@@ -12361,7 +12361,7 @@
       <c r="D133" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E133" s="16" t="n">
+      <c r="E133" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F133" s="20" t="n">
@@ -12394,7 +12394,7 @@
       <c r="D134" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E134" s="16" t="n">
+      <c r="E134" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F134" s="20" t="n">
@@ -12427,7 +12427,7 @@
       <c r="D135" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E135" s="16" t="n">
+      <c r="E135" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F135" s="20" t="n">
@@ -12460,7 +12460,7 @@
       <c r="D136" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E136" s="16" t="n">
+      <c r="E136" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F136" s="20" t="n">
@@ -12493,7 +12493,7 @@
       <c r="D137" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E137" s="16" t="n">
+      <c r="E137" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F137" s="20" t="n">
@@ -12526,7 +12526,7 @@
       <c r="D138" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E138" s="16" t="n">
+      <c r="E138" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F138" s="20" t="n">
@@ -12559,7 +12559,7 @@
       <c r="D139" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E139" s="16" t="n">
+      <c r="E139" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F139" s="20" t="n">
@@ -12592,7 +12592,7 @@
       <c r="D140" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E140" s="16" t="n">
+      <c r="E140" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F140" s="20" t="n">
@@ -12625,7 +12625,7 @@
       <c r="D141" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E141" s="16" t="n">
+      <c r="E141" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F141" s="20" t="n">
@@ -12658,7 +12658,7 @@
       <c r="D142" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E142" s="16" t="n">
+      <c r="E142" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F142" s="20" t="n">
@@ -12691,7 +12691,7 @@
       <c r="D143" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E143" s="16" t="n">
+      <c r="E143" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F143" s="20" t="n">
@@ -12724,7 +12724,7 @@
       <c r="D144" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E144" s="16" t="n">
+      <c r="E144" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F144" s="20" t="n">
@@ -12757,7 +12757,7 @@
       <c r="D145" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E145" s="16" t="n">
+      <c r="E145" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F145" s="20" t="n">
@@ -12790,7 +12790,7 @@
       <c r="D146" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E146" s="16" t="n">
+      <c r="E146" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F146" s="20" t="n">
@@ -12823,7 +12823,7 @@
       <c r="D147" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E147" s="16" t="n">
+      <c r="E147" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F147" s="20" t="n">
@@ -12856,7 +12856,7 @@
       <c r="D148" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E148" s="16" t="n">
+      <c r="E148" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F148" s="20" t="n">
@@ -12889,7 +12889,7 @@
       <c r="D149" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E149" s="16" t="n">
+      <c r="E149" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F149" s="20" t="n">
@@ -12922,7 +12922,7 @@
       <c r="D150" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E150" s="16" t="n">
+      <c r="E150" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F150" s="20" t="n">
@@ -12955,7 +12955,7 @@
       <c r="D151" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E151" s="16" t="n">
+      <c r="E151" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F151" s="20" t="n">
@@ -12988,7 +12988,7 @@
       <c r="D152" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E152" s="16" t="n">
+      <c r="E152" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F152" s="20" t="n">
@@ -13021,7 +13021,7 @@
       <c r="D153" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E153" s="16" t="n">
+      <c r="E153" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F153" s="20" t="n">
@@ -13054,7 +13054,7 @@
       <c r="D154" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E154" s="16" t="n">
+      <c r="E154" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F154" s="20" t="n">
@@ -13091,7 +13091,7 @@
       <c r="D155" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E155" s="16" t="n">
+      <c r="E155" s="12" t="n">
         <v>1.0443</v>
       </c>
       <c r="F155" s="20" t="n">
@@ -13124,7 +13124,7 @@
       <c r="D156" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E156" s="17" t="n">
+      <c r="E156" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F156" s="21" t="n">
@@ -13157,7 +13157,7 @@
       <c r="D157" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E157" s="16" t="n">
+      <c r="E157" s="12" t="n">
         <v>1.008</v>
       </c>
       <c r="F157" s="20" t="n">
@@ -13190,7 +13190,7 @@
       <c r="D158" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E158" s="16" t="n">
+      <c r="E158" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F158" s="20" t="n">
@@ -13223,7 +13223,7 @@
       <c r="D159" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E159" s="16" t="n">
+      <c r="E159" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F159" s="20" t="n">
@@ -13256,7 +13256,7 @@
       <c r="D160" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E160" s="16" t="n">
+      <c r="E160" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F160" s="20" t="n">
@@ -13289,7 +13289,7 @@
       <c r="D161" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E161" s="16" t="n">
+      <c r="E161" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F161" s="20" t="n">
@@ -13322,7 +13322,7 @@
       <c r="D162" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E162" s="16" t="n">
+      <c r="E162" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F162" s="20" t="n">
@@ -13355,7 +13355,7 @@
       <c r="D163" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E163" s="16" t="n">
+      <c r="E163" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F163" s="20" t="n">
@@ -13388,7 +13388,7 @@
       <c r="D164" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E164" s="16" t="n">
+      <c r="E164" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F164" s="20" t="n">
@@ -13421,7 +13421,7 @@
       <c r="D165" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E165" s="16" t="n">
+      <c r="E165" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F165" s="20" t="n">
@@ -13454,7 +13454,7 @@
       <c r="D166" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E166" s="16" t="n">
+      <c r="E166" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F166" s="20" t="n">
@@ -13487,7 +13487,7 @@
       <c r="D167" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E167" s="16" t="n">
+      <c r="E167" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F167" s="20" t="n">
@@ -13520,7 +13520,7 @@
       <c r="D168" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E168" s="16" t="n">
+      <c r="E168" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F168" s="20" t="n">
@@ -13553,7 +13553,7 @@
       <c r="D169" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E169" s="16" t="n">
+      <c r="E169" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F169" s="20" t="n">
@@ -13586,7 +13586,7 @@
       <c r="D170" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E170" s="16" t="n">
+      <c r="E170" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F170" s="20" t="n">
@@ -13619,7 +13619,7 @@
       <c r="D171" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E171" s="16" t="n">
+      <c r="E171" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F171" s="20" t="n">
@@ -13652,7 +13652,7 @@
       <c r="D172" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E172" s="16" t="n">
+      <c r="E172" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F172" s="20" t="n">
@@ -13685,7 +13685,7 @@
       <c r="D173" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E173" s="16" t="n">
+      <c r="E173" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F173" s="20" t="n">
@@ -13718,7 +13718,7 @@
       <c r="D174" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E174" s="16" t="n">
+      <c r="E174" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F174" s="20" t="n">
@@ -13751,7 +13751,7 @@
       <c r="D175" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E175" s="16" t="n">
+      <c r="E175" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F175" s="20" t="n">
@@ -13784,7 +13784,7 @@
       <c r="D176" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E176" s="16" t="n">
+      <c r="E176" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F176" s="20" t="n">
@@ -13817,7 +13817,7 @@
       <c r="D177" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E177" s="16" t="n">
+      <c r="E177" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F177" s="20" t="n">
@@ -13850,7 +13850,7 @@
       <c r="D178" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E178" s="16" t="n">
+      <c r="E178" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F178" s="20" t="n">
@@ -13883,7 +13883,7 @@
       <c r="D179" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E179" s="16" t="n">
+      <c r="E179" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F179" s="20" t="n">
@@ -13920,7 +13920,7 @@
       <c r="D180" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E180" s="16" t="n">
+      <c r="E180" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F180" s="20" t="n">
@@ -13953,7 +13953,7 @@
       <c r="D181" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="E181" s="16" t="n">
+      <c r="E181" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F181" s="20" t="n">
@@ -13986,7 +13986,7 @@
       <c r="D182" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E182" s="16" t="n">
+      <c r="E182" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F182" s="20" t="n">
@@ -14019,7 +14019,7 @@
       <c r="D183" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E183" s="16" t="n">
+      <c r="E183" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F183" s="20" t="n">
@@ -14052,7 +14052,7 @@
       <c r="D184" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E184" s="17" t="n">
+      <c r="E184" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F184" s="21" t="n">
@@ -14085,7 +14085,7 @@
       <c r="D185" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E185" s="16" t="n">
+      <c r="E185" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F185" s="20" t="n">
@@ -14118,7 +14118,7 @@
       <c r="D186" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E186" s="16" t="n">
+      <c r="E186" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F186" s="20" t="n">
@@ -14151,7 +14151,7 @@
       <c r="D187" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E187" s="16" t="n">
+      <c r="E187" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F187" s="20" t="n">
@@ -14184,7 +14184,7 @@
       <c r="D188" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E188" s="16" t="n">
+      <c r="E188" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F188" s="20" t="n">
@@ -14217,7 +14217,7 @@
       <c r="D189" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E189" s="16" t="n">
+      <c r="E189" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F189" s="20" t="n">
@@ -14250,7 +14250,7 @@
       <c r="D190" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E190" s="16" t="n">
+      <c r="E190" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F190" s="20" t="n">
@@ -14283,7 +14283,7 @@
       <c r="D191" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E191" s="16" t="n">
+      <c r="E191" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F191" s="20" t="n">
@@ -14316,7 +14316,7 @@
       <c r="D192" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E192" s="16" t="n">
+      <c r="E192" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F192" s="20" t="n">
@@ -14349,7 +14349,7 @@
       <c r="D193" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E193" s="16" t="n">
+      <c r="E193" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F193" s="20" t="n">
@@ -14382,7 +14382,7 @@
       <c r="D194" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E194" s="16" t="n">
+      <c r="E194" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F194" s="20" t="n">
@@ -14415,7 +14415,7 @@
       <c r="D195" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E195" s="16" t="n">
+      <c r="E195" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F195" s="20" t="n">
@@ -14448,7 +14448,7 @@
       <c r="D196" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E196" s="16" t="n">
+      <c r="E196" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F196" s="20" t="n">
@@ -14481,7 +14481,7 @@
       <c r="D197" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E197" s="16" t="n">
+      <c r="E197" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F197" s="20" t="n">
@@ -14514,7 +14514,7 @@
       <c r="D198" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E198" s="16" t="n">
+      <c r="E198" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F198" s="20" t="n">
@@ -14547,7 +14547,7 @@
       <c r="D199" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E199" s="16" t="n">
+      <c r="E199" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F199" s="20" t="n">
@@ -14580,7 +14580,7 @@
       <c r="D200" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E200" s="16" t="n">
+      <c r="E200" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F200" s="20" t="n">
@@ -14613,7 +14613,7 @@
       <c r="D201" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E201" s="16" t="n">
+      <c r="E201" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F201" s="20" t="n">
@@ -14646,7 +14646,7 @@
       <c r="D202" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E202" s="16" t="n">
+      <c r="E202" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F202" s="20" t="n">
@@ -14679,7 +14679,7 @@
       <c r="D203" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E203" s="16" t="n">
+      <c r="E203" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F203" s="20" t="n">
@@ -14712,7 +14712,7 @@
       <c r="D204" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E204" s="16" t="n">
+      <c r="E204" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F204" s="20" t="n">
@@ -14749,7 +14749,7 @@
       <c r="D205" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E205" s="17" t="n">
+      <c r="E205" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F205" s="21" t="n">
@@ -14782,7 +14782,7 @@
       <c r="D206" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E206" s="16" t="n">
+      <c r="E206" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F206" s="20" t="n">
@@ -14815,7 +14815,7 @@
       <c r="D207" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E207" s="16" t="n">
+      <c r="E207" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F207" s="20" t="n">
@@ -14848,7 +14848,7 @@
       <c r="D208" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="E208" s="16" t="n">
+      <c r="E208" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F208" s="20" t="n">
@@ -14881,7 +14881,7 @@
       <c r="D209" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E209" s="16" t="n">
+      <c r="E209" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F209" s="20" t="n">
@@ -14914,7 +14914,7 @@
       <c r="D210" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E210" s="16" t="n">
+      <c r="E210" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F210" s="20" t="n">
@@ -14947,7 +14947,7 @@
       <c r="D211" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E211" s="16" t="n">
+      <c r="E211" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F211" s="20" t="n">
@@ -14980,7 +14980,7 @@
       <c r="D212" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E212" s="16" t="n">
+      <c r="E212" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F212" s="20" t="n">
@@ -15013,7 +15013,7 @@
       <c r="D213" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E213" s="16" t="n">
+      <c r="E213" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F213" s="20" t="n">
@@ -15046,7 +15046,7 @@
       <c r="D214" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E214" s="16" t="n">
+      <c r="E214" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F214" s="20" t="n">
@@ -15079,7 +15079,7 @@
       <c r="D215" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E215" s="16" t="n">
+      <c r="E215" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F215" s="20" t="n">
@@ -15112,7 +15112,7 @@
       <c r="D216" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E216" s="16" t="n">
+      <c r="E216" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F216" s="20" t="n">
@@ -15145,7 +15145,7 @@
       <c r="D217" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E217" s="16" t="n">
+      <c r="E217" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F217" s="20" t="n">
@@ -15178,7 +15178,7 @@
       <c r="D218" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E218" s="16" t="n">
+      <c r="E218" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F218" s="20" t="n">
@@ -15211,7 +15211,7 @@
       <c r="D219" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E219" s="16" t="n">
+      <c r="E219" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F219" s="20" t="n">
@@ -15244,7 +15244,7 @@
       <c r="D220" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E220" s="16" t="n">
+      <c r="E220" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F220" s="20" t="n">
@@ -15277,7 +15277,7 @@
       <c r="D221" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E221" s="16" t="n">
+      <c r="E221" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F221" s="20" t="n">
@@ -15310,7 +15310,7 @@
       <c r="D222" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E222" s="16" t="n">
+      <c r="E222" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F222" s="20" t="n">
@@ -15343,7 +15343,7 @@
       <c r="D223" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E223" s="16" t="n">
+      <c r="E223" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F223" s="20" t="n">
@@ -15376,7 +15376,7 @@
       <c r="D224" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E224" s="16" t="n">
+      <c r="E224" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F224" s="20" t="n">
@@ -15409,7 +15409,7 @@
       <c r="D225" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E225" s="16" t="n">
+      <c r="E225" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F225" s="20" t="n">
@@ -15442,7 +15442,7 @@
       <c r="D226" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E226" s="16" t="n">
+      <c r="E226" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F226" s="20" t="n">
@@ -15475,7 +15475,7 @@
       <c r="D227" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E227" s="16" t="n">
+      <c r="E227" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F227" s="20" t="n">
@@ -15508,7 +15508,7 @@
       <c r="D228" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E228" s="16" t="n">
+      <c r="E228" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F228" s="20" t="n">
@@ -15541,7 +15541,7 @@
       <c r="D229" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E229" s="16" t="n">
+      <c r="E229" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F229" s="20" t="n">
@@ -15578,7 +15578,7 @@
       <c r="D230" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E230" s="17" t="n">
+      <c r="E230" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F230" s="21" t="n">
@@ -15611,7 +15611,7 @@
       <c r="D231" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="E231" s="16" t="n">
+      <c r="E231" s="12" t="n">
         <v>0.388</v>
       </c>
       <c r="F231" s="20" t="n">
@@ -15644,7 +15644,7 @@
       <c r="D232" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E232" s="16" t="n">
+      <c r="E232" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F232" s="20" t="n">
@@ -15677,7 +15677,7 @@
       <c r="D233" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E233" s="16" t="n">
+      <c r="E233" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F233" s="20" t="n">
@@ -15710,7 +15710,7 @@
       <c r="D234" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E234" s="16" t="n">
+      <c r="E234" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F234" s="20" t="n">
@@ -15743,7 +15743,7 @@
       <c r="D235" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E235" s="16" t="n">
+      <c r="E235" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F235" s="20" t="n">
@@ -15776,7 +15776,7 @@
       <c r="D236" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E236" s="16" t="n">
+      <c r="E236" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F236" s="20" t="n">
@@ -15809,7 +15809,7 @@
       <c r="D237" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E237" s="16" t="n">
+      <c r="E237" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F237" s="20" t="n">
@@ -15842,7 +15842,7 @@
       <c r="D238" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E238" s="16" t="n">
+      <c r="E238" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F238" s="20" t="n">
@@ -15875,7 +15875,7 @@
       <c r="D239" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E239" s="16" t="n">
+      <c r="E239" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F239" s="20" t="n">
@@ -15908,7 +15908,7 @@
       <c r="D240" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E240" s="16" t="n">
+      <c r="E240" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F240" s="20" t="n">
@@ -15941,7 +15941,7 @@
       <c r="D241" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E241" s="16" t="n">
+      <c r="E241" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F241" s="20" t="n">
@@ -15974,7 +15974,7 @@
       <c r="D242" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E242" s="16" t="n">
+      <c r="E242" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F242" s="20" t="n">
@@ -16007,7 +16007,7 @@
       <c r="D243" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E243" s="16" t="n">
+      <c r="E243" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F243" s="20" t="n">
@@ -16040,7 +16040,7 @@
       <c r="D244" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E244" s="16" t="n">
+      <c r="E244" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F244" s="20" t="n">
@@ -16073,7 +16073,7 @@
       <c r="D245" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E245" s="16" t="n">
+      <c r="E245" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F245" s="20" t="n">
@@ -16106,7 +16106,7 @@
       <c r="D246" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E246" s="16" t="n">
+      <c r="E246" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F246" s="20" t="n">
@@ -16139,7 +16139,7 @@
       <c r="D247" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E247" s="16" t="n">
+      <c r="E247" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F247" s="20" t="n">
@@ -16172,7 +16172,7 @@
       <c r="D248" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E248" s="16" t="n">
+      <c r="E248" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F248" s="20" t="n">
@@ -16205,7 +16205,7 @@
       <c r="D249" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E249" s="16" t="n">
+      <c r="E249" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F249" s="20" t="n">
@@ -16238,7 +16238,7 @@
       <c r="D250" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E250" s="16" t="n">
+      <c r="E250" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F250" s="20" t="n">
@@ -16271,7 +16271,7 @@
       <c r="D251" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E251" s="16" t="n">
+      <c r="E251" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F251" s="20" t="n">
@@ -16304,7 +16304,7 @@
       <c r="D252" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E252" s="16" t="n">
+      <c r="E252" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F252" s="20" t="n">
@@ -16337,7 +16337,7 @@
       <c r="D253" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E253" s="16" t="n">
+      <c r="E253" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F253" s="20" t="n">
@@ -16370,7 +16370,7 @@
       <c r="D254" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E254" s="16" t="n">
+      <c r="E254" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F254" s="20" t="n">
@@ -16407,7 +16407,7 @@
       <c r="D255" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E255" s="17" t="n">
+      <c r="E255" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F255" s="21" t="n">
@@ -16440,7 +16440,7 @@
       <c r="D256" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E256" s="16" t="n">
+      <c r="E256" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F256" s="20" t="n">
@@ -16473,7 +16473,7 @@
       <c r="D257" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E257" s="16" t="n">
+      <c r="E257" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F257" s="20" t="n">
@@ -16506,7 +16506,7 @@
       <c r="D258" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E258" s="16" t="n">
+      <c r="E258" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F258" s="20" t="n">
@@ -16539,7 +16539,7 @@
       <c r="D259" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E259" s="16" t="n">
+      <c r="E259" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F259" s="20" t="n">
@@ -16572,7 +16572,7 @@
       <c r="D260" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E260" s="16" t="n">
+      <c r="E260" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F260" s="20" t="n">
@@ -16605,7 +16605,7 @@
       <c r="D261" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E261" s="16" t="n">
+      <c r="E261" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F261" s="20" t="n">
@@ -16638,7 +16638,7 @@
       <c r="D262" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E262" s="16" t="n">
+      <c r="E262" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F262" s="20" t="n">
@@ -16671,7 +16671,7 @@
       <c r="D263" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E263" s="16" t="n">
+      <c r="E263" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F263" s="20" t="n">
@@ -16704,7 +16704,7 @@
       <c r="D264" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E264" s="16" t="n">
+      <c r="E264" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F264" s="20" t="n">
@@ -16737,7 +16737,7 @@
       <c r="D265" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E265" s="16" t="n">
+      <c r="E265" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F265" s="20" t="n">
@@ -16770,7 +16770,7 @@
       <c r="D266" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E266" s="16" t="n">
+      <c r="E266" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F266" s="20" t="n">
@@ -16803,7 +16803,7 @@
       <c r="D267" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E267" s="16" t="n">
+      <c r="E267" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F267" s="20" t="n">
@@ -16836,7 +16836,7 @@
       <c r="D268" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E268" s="16" t="n">
+      <c r="E268" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F268" s="20" t="n">
@@ -16869,7 +16869,7 @@
       <c r="D269" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E269" s="16" t="n">
+      <c r="E269" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F269" s="20" t="n">
@@ -16902,7 +16902,7 @@
       <c r="D270" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E270" s="16" t="n">
+      <c r="E270" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F270" s="20" t="n">
@@ -16935,7 +16935,7 @@
       <c r="D271" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E271" s="16" t="n">
+      <c r="E271" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F271" s="20" t="n">
@@ -16968,7 +16968,7 @@
       <c r="D272" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E272" s="16" t="n">
+      <c r="E272" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F272" s="20" t="n">
@@ -17001,7 +17001,7 @@
       <c r="D273" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E273" s="16" t="n">
+      <c r="E273" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F273" s="20" t="n">
@@ -17034,7 +17034,7 @@
       <c r="D274" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E274" s="16" t="n">
+      <c r="E274" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F274" s="20" t="n">
@@ -17067,7 +17067,7 @@
       <c r="D275" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E275" s="16" t="n">
+      <c r="E275" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F275" s="20" t="n">
@@ -17100,7 +17100,7 @@
       <c r="D276" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E276" s="16" t="n">
+      <c r="E276" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F276" s="20" t="n">
@@ -17133,7 +17133,7 @@
       <c r="D277" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E277" s="16" t="n">
+      <c r="E277" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F277" s="20" t="n">
@@ -17166,7 +17166,7 @@
       <c r="D278" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E278" s="16" t="n">
+      <c r="E278" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F278" s="20" t="n">
@@ -17199,7 +17199,7 @@
       <c r="D279" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E279" s="16" t="n">
+      <c r="E279" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F279" s="20" t="n">
@@ -17236,7 +17236,7 @@
       <c r="D280" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="E280" s="16" t="n">
+      <c r="E280" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F280" s="20" t="n">
@@ -17269,7 +17269,7 @@
       <c r="D281" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="E281" s="16" t="n">
+      <c r="E281" s="12" t="n">
         <v>1.4125</v>
       </c>
       <c r="F281" s="20" t="n">
@@ -17302,7 +17302,7 @@
       <c r="D282" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="E282" s="16" t="n">
+      <c r="E282" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F282" s="20" t="n">
@@ -17335,7 +17335,7 @@
       <c r="D283" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E283" s="16" t="n">
+      <c r="E283" s="12" t="n">
         <v>1.6934</v>
       </c>
       <c r="F283" s="20" t="n">
@@ -17368,7 +17368,7 @@
       <c r="D284" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E284" s="16" t="n">
+      <c r="E284" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F284" s="20" t="n">
@@ -17401,7 +17401,7 @@
       <c r="D285" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E285" s="17" t="n">
+      <c r="E285" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F285" s="21" t="n">
@@ -17434,7 +17434,7 @@
       <c r="D286" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E286" s="16" t="n">
+      <c r="E286" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F286" s="20" t="n">
@@ -17467,7 +17467,7 @@
       <c r="D287" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E287" s="16" t="n">
+      <c r="E287" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F287" s="20" t="n">
@@ -17500,7 +17500,7 @@
       <c r="D288" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E288" s="16" t="n">
+      <c r="E288" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F288" s="20" t="n">
@@ -17533,7 +17533,7 @@
       <c r="D289" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E289" s="16" t="n">
+      <c r="E289" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F289" s="20" t="n">
@@ -17566,7 +17566,7 @@
       <c r="D290" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E290" s="16" t="n">
+      <c r="E290" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F290" s="20" t="n">
@@ -17599,7 +17599,7 @@
       <c r="D291" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E291" s="16" t="n">
+      <c r="E291" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F291" s="20" t="n">
@@ -17632,7 +17632,7 @@
       <c r="D292" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E292" s="16" t="n">
+      <c r="E292" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F292" s="20" t="n">
@@ -17665,7 +17665,7 @@
       <c r="D293" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E293" s="16" t="n">
+      <c r="E293" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F293" s="20" t="n">
@@ -17698,7 +17698,7 @@
       <c r="D294" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E294" s="16" t="n">
+      <c r="E294" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F294" s="20" t="n">
@@ -17731,7 +17731,7 @@
       <c r="D295" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E295" s="16" t="n">
+      <c r="E295" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F295" s="20" t="n">
@@ -17764,7 +17764,7 @@
       <c r="D296" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E296" s="16" t="n">
+      <c r="E296" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F296" s="20" t="n">
@@ -17797,7 +17797,7 @@
       <c r="D297" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E297" s="16" t="n">
+      <c r="E297" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F297" s="20" t="n">
@@ -17830,7 +17830,7 @@
       <c r="D298" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E298" s="16" t="n">
+      <c r="E298" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F298" s="20" t="n">
@@ -17863,7 +17863,7 @@
       <c r="D299" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E299" s="16" t="n">
+      <c r="E299" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F299" s="20" t="n">
@@ -17896,7 +17896,7 @@
       <c r="D300" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E300" s="16" t="n">
+      <c r="E300" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F300" s="20" t="n">
@@ -17929,7 +17929,7 @@
       <c r="D301" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E301" s="16" t="n">
+      <c r="E301" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F301" s="20" t="n">
@@ -17962,7 +17962,7 @@
       <c r="D302" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E302" s="16" t="n">
+      <c r="E302" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F302" s="20" t="n">
@@ -17995,7 +17995,7 @@
       <c r="D303" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E303" s="16" t="n">
+      <c r="E303" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F303" s="20" t="n">
@@ -18028,7 +18028,7 @@
       <c r="D304" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E304" s="16" t="n">
+      <c r="E304" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F304" s="20" t="n">
@@ -18065,7 +18065,7 @@
       <c r="D305" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E305" s="17" t="n">
+      <c r="E305" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F305" s="21" t="n">
@@ -18098,7 +18098,7 @@
       <c r="D306" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E306" s="16" t="n">
+      <c r="E306" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F306" s="20" t="n">
@@ -18131,7 +18131,7 @@
       <c r="D307" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E307" s="16" t="n">
+      <c r="E307" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F307" s="20" t="n">
@@ -18164,7 +18164,7 @@
       <c r="D308" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E308" s="16" t="n">
+      <c r="E308" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F308" s="20" t="n">
@@ -18197,7 +18197,7 @@
       <c r="D309" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E309" s="16" t="n">
+      <c r="E309" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F309" s="20" t="n">
@@ -18230,7 +18230,7 @@
       <c r="D310" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E310" s="16" t="n">
+      <c r="E310" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F310" s="20" t="n">
@@ -18263,7 +18263,7 @@
       <c r="D311" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E311" s="16" t="n">
+      <c r="E311" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F311" s="20" t="n">
@@ -18296,7 +18296,7 @@
       <c r="D312" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E312" s="16" t="n">
+      <c r="E312" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F312" s="20" t="n">
@@ -18329,7 +18329,7 @@
       <c r="D313" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E313" s="16" t="n">
+      <c r="E313" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F313" s="20" t="n">
@@ -18362,7 +18362,7 @@
       <c r="D314" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E314" s="16" t="n">
+      <c r="E314" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F314" s="20" t="n">
@@ -18395,7 +18395,7 @@
       <c r="D315" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E315" s="16" t="n">
+      <c r="E315" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F315" s="20" t="n">
@@ -18428,7 +18428,7 @@
       <c r="D316" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E316" s="16" t="n">
+      <c r="E316" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F316" s="20" t="n">
@@ -18461,7 +18461,7 @@
       <c r="D317" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E317" s="16" t="n">
+      <c r="E317" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F317" s="20" t="n">
@@ -18494,7 +18494,7 @@
       <c r="D318" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E318" s="16" t="n">
+      <c r="E318" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F318" s="20" t="n">
@@ -18527,7 +18527,7 @@
       <c r="D319" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E319" s="16" t="n">
+      <c r="E319" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F319" s="20" t="n">
@@ -18560,7 +18560,7 @@
       <c r="D320" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E320" s="16" t="n">
+      <c r="E320" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F320" s="20" t="n">
@@ -18593,7 +18593,7 @@
       <c r="D321" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E321" s="16" t="n">
+      <c r="E321" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F321" s="20" t="n">
@@ -18626,7 +18626,7 @@
       <c r="D322" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E322" s="16" t="n">
+      <c r="E322" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F322" s="20" t="n">
@@ -18659,7 +18659,7 @@
       <c r="D323" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E323" s="16" t="n">
+      <c r="E323" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F323" s="20" t="n">
@@ -18692,7 +18692,7 @@
       <c r="D324" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E324" s="16" t="n">
+      <c r="E324" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F324" s="20" t="n">
@@ -18725,7 +18725,7 @@
       <c r="D325" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E325" s="16" t="n">
+      <c r="E325" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F325" s="20" t="n">
@@ -18758,7 +18758,7 @@
       <c r="D326" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E326" s="16" t="n">
+      <c r="E326" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F326" s="20" t="n">
@@ -18791,7 +18791,7 @@
       <c r="D327" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E327" s="16" t="n">
+      <c r="E327" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F327" s="20" t="n">
@@ -18824,7 +18824,7 @@
       <c r="D328" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E328" s="16" t="n">
+      <c r="E328" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F328" s="20" t="n">
@@ -18857,7 +18857,7 @@
       <c r="D329" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E329" s="16" t="n">
+      <c r="E329" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F329" s="20" t="n">
@@ -18894,7 +18894,7 @@
       <c r="D330" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E330" s="16" t="n">
+      <c r="E330" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F330" s="20" t="n">
@@ -18927,7 +18927,7 @@
       <c r="D331" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="E331" s="16" t="n">
+      <c r="E331" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F331" s="20" t="n">
@@ -18960,7 +18960,7 @@
       <c r="D332" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E332" s="17" t="n">
+      <c r="E332" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F332" s="21" t="n">
@@ -18993,7 +18993,7 @@
       <c r="D333" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E333" s="16" t="n">
+      <c r="E333" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F333" s="20" t="n">
@@ -19026,7 +19026,7 @@
       <c r="D334" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E334" s="16" t="n">
+      <c r="E334" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F334" s="20" t="n">
@@ -19059,7 +19059,7 @@
       <c r="D335" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E335" s="16" t="n">
+      <c r="E335" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F335" s="20" t="n">
@@ -19092,7 +19092,7 @@
       <c r="D336" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E336" s="16" t="n">
+      <c r="E336" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F336" s="20" t="n">
@@ -19125,7 +19125,7 @@
       <c r="D337" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E337" s="16" t="n">
+      <c r="E337" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F337" s="20" t="n">
@@ -19158,7 +19158,7 @@
       <c r="D338" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E338" s="16" t="n">
+      <c r="E338" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F338" s="20" t="n">
@@ -19191,7 +19191,7 @@
       <c r="D339" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E339" s="16" t="n">
+      <c r="E339" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F339" s="20" t="n">
@@ -19224,7 +19224,7 @@
       <c r="D340" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E340" s="16" t="n">
+      <c r="E340" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F340" s="20" t="n">
@@ -19257,7 +19257,7 @@
       <c r="D341" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E341" s="16" t="n">
+      <c r="E341" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F341" s="20" t="n">
@@ -19290,7 +19290,7 @@
       <c r="D342" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E342" s="16" t="n">
+      <c r="E342" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F342" s="20" t="n">
@@ -19323,7 +19323,7 @@
       <c r="D343" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E343" s="16" t="n">
+      <c r="E343" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F343" s="20" t="n">
@@ -19356,7 +19356,7 @@
       <c r="D344" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E344" s="16" t="n">
+      <c r="E344" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F344" s="20" t="n">
@@ -19389,7 +19389,7 @@
       <c r="D345" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E345" s="16" t="n">
+      <c r="E345" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F345" s="20" t="n">
@@ -19422,7 +19422,7 @@
       <c r="D346" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E346" s="16" t="n">
+      <c r="E346" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F346" s="20" t="n">
@@ -19455,7 +19455,7 @@
       <c r="D347" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E347" s="16" t="n">
+      <c r="E347" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F347" s="20" t="n">
@@ -19488,7 +19488,7 @@
       <c r="D348" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="E348" s="16" t="n">
+      <c r="E348" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F348" s="20" t="n">
@@ -19521,7 +19521,7 @@
       <c r="D349" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E349" s="16" t="n">
+      <c r="E349" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F349" s="20" t="n">
@@ -19554,7 +19554,7 @@
       <c r="D350" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E350" s="16" t="n">
+      <c r="E350" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F350" s="20" t="n">
@@ -19587,7 +19587,7 @@
       <c r="D351" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E351" s="16" t="n">
+      <c r="E351" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F351" s="20" t="n">
@@ -19620,7 +19620,7 @@
       <c r="D352" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E352" s="16" t="n">
+      <c r="E352" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F352" s="20" t="n">
@@ -19653,7 +19653,7 @@
       <c r="D353" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E353" s="16" t="n">
+      <c r="E353" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F353" s="20" t="n">
@@ -19686,7 +19686,7 @@
       <c r="D354" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E354" s="16" t="n">
+      <c r="E354" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F354" s="20" t="n">
@@ -19723,7 +19723,7 @@
       <c r="D355" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E355" s="16" t="n">
+      <c r="E355" s="12" t="n">
         <v>0.835</v>
       </c>
       <c r="F355" s="20" t="n">
@@ -19756,7 +19756,7 @@
       <c r="D356" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E356" s="16" t="n">
+      <c r="E356" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F356" s="20" t="n">
@@ -19789,7 +19789,7 @@
       <c r="D357" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E357" s="17" t="n">
+      <c r="E357" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F357" s="21" t="n">
@@ -19822,7 +19822,7 @@
       <c r="D358" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E358" s="16" t="n">
+      <c r="E358" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F358" s="20" t="n">
@@ -19855,7 +19855,7 @@
       <c r="D359" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E359" s="16" t="n">
+      <c r="E359" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F359" s="20" t="n">
@@ -19888,7 +19888,7 @@
       <c r="D360" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E360" s="16" t="n">
+      <c r="E360" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F360" s="20" t="n">
@@ -19921,7 +19921,7 @@
       <c r="D361" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E361" s="16" t="n">
+      <c r="E361" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F361" s="20" t="n">
@@ -19954,7 +19954,7 @@
       <c r="D362" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E362" s="16" t="n">
+      <c r="E362" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F362" s="20" t="n">
@@ -19987,7 +19987,7 @@
       <c r="D363" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E363" s="16" t="n">
+      <c r="E363" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F363" s="20" t="n">
@@ -20020,7 +20020,7 @@
       <c r="D364" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E364" s="16" t="n">
+      <c r="E364" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F364" s="20" t="n">
@@ -20053,7 +20053,7 @@
       <c r="D365" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E365" s="16" t="n">
+      <c r="E365" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F365" s="20" t="n">
@@ -20086,7 +20086,7 @@
       <c r="D366" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E366" s="16" t="n">
+      <c r="E366" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F366" s="20" t="n">
@@ -20119,7 +20119,7 @@
       <c r="D367" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E367" s="16" t="n">
+      <c r="E367" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F367" s="20" t="n">
@@ -20152,7 +20152,7 @@
       <c r="D368" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E368" s="16" t="n">
+      <c r="E368" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F368" s="20" t="n">
@@ -20185,7 +20185,7 @@
       <c r="D369" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E369" s="16" t="n">
+      <c r="E369" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F369" s="20" t="n">
@@ -20218,7 +20218,7 @@
       <c r="D370" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E370" s="16" t="n">
+      <c r="E370" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F370" s="20" t="n">
@@ -20251,7 +20251,7 @@
       <c r="D371" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E371" s="16" t="n">
+      <c r="E371" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F371" s="20" t="n">
@@ -20284,7 +20284,7 @@
       <c r="D372" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E372" s="16" t="n">
+      <c r="E372" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F372" s="20" t="n">
@@ -20317,7 +20317,7 @@
       <c r="D373" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E373" s="16" t="n">
+      <c r="E373" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F373" s="20" t="n">
@@ -20350,7 +20350,7 @@
       <c r="D374" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E374" s="16" t="n">
+      <c r="E374" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F374" s="20" t="n">
@@ -20383,7 +20383,7 @@
       <c r="D375" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E375" s="16" t="n">
+      <c r="E375" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F375" s="20" t="n">
@@ -20416,7 +20416,7 @@
       <c r="D376" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E376" s="16" t="n">
+      <c r="E376" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F376" s="20" t="n">
@@ -20449,7 +20449,7 @@
       <c r="D377" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E377" s="16" t="n">
+      <c r="E377" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F377" s="20" t="n">
@@ -20482,7 +20482,7 @@
       <c r="D378" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E378" s="16" t="n">
+      <c r="E378" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F378" s="20" t="n">
@@ -20515,7 +20515,7 @@
       <c r="D379" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E379" s="16" t="n">
+      <c r="E379" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F379" s="20" t="n">
@@ -20552,7 +20552,7 @@
       <c r="D380" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E380" s="16" t="n">
+      <c r="E380" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F380" s="20" t="n">
@@ -20585,7 +20585,7 @@
       <c r="D381" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E381" s="16" t="n">
+      <c r="E381" s="12" t="n">
         <v>0.6614</v>
       </c>
       <c r="F381" s="20" t="n">
@@ -20618,7 +20618,7 @@
       <c r="D382" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E382" s="16" t="n">
+      <c r="E382" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F382" s="20" t="n">
@@ -20651,7 +20651,7 @@
       <c r="D383" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E383" s="16" t="n">
+      <c r="E383" s="12" t="n">
         <v>1.2078</v>
       </c>
       <c r="F383" s="20" t="n">
@@ -20684,7 +20684,7 @@
       <c r="D384" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E384" s="16" t="n">
+      <c r="E384" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F384" s="20" t="n">
@@ -20717,7 +20717,7 @@
       <c r="D385" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E385" s="16" t="n">
+      <c r="E385" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F385" s="20" t="n">
@@ -20750,7 +20750,7 @@
       <c r="D386" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E386" s="17" t="n">
+      <c r="E386" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F386" s="21" t="n">
@@ -20783,7 +20783,7 @@
       <c r="D387" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E387" s="16" t="n">
+      <c r="E387" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F387" s="20" t="n">
@@ -20816,7 +20816,7 @@
       <c r="D388" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E388" s="16" t="n">
+      <c r="E388" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F388" s="20" t="n">
@@ -20849,7 +20849,7 @@
       <c r="D389" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E389" s="16" t="n">
+      <c r="E389" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F389" s="20" t="n">
@@ -20882,7 +20882,7 @@
       <c r="D390" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E390" s="16" t="n">
+      <c r="E390" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F390" s="20" t="n">
@@ -20915,7 +20915,7 @@
       <c r="D391" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E391" s="16" t="n">
+      <c r="E391" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F391" s="20" t="n">
@@ -20948,7 +20948,7 @@
       <c r="D392" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E392" s="16" t="n">
+      <c r="E392" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F392" s="20" t="n">
@@ -20981,7 +20981,7 @@
       <c r="D393" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E393" s="16" t="n">
+      <c r="E393" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F393" s="20" t="n">
@@ -21014,7 +21014,7 @@
       <c r="D394" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E394" s="16" t="n">
+      <c r="E394" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F394" s="20" t="n">
@@ -21047,7 +21047,7 @@
       <c r="D395" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E395" s="16" t="n">
+      <c r="E395" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F395" s="20" t="n">
@@ -21080,7 +21080,7 @@
       <c r="D396" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E396" s="16" t="n">
+      <c r="E396" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F396" s="20" t="n">
@@ -21113,7 +21113,7 @@
       <c r="D397" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E397" s="16" t="n">
+      <c r="E397" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F397" s="20" t="n">
@@ -21146,7 +21146,7 @@
       <c r="D398" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E398" s="16" t="n">
+      <c r="E398" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F398" s="20" t="n">
@@ -21179,7 +21179,7 @@
       <c r="D399" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E399" s="16" t="n">
+      <c r="E399" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F399" s="20" t="n">
@@ -21212,7 +21212,7 @@
       <c r="D400" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E400" s="16" t="n">
+      <c r="E400" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F400" s="20" t="n">
@@ -21245,7 +21245,7 @@
       <c r="D401" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E401" s="16" t="n">
+      <c r="E401" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F401" s="20" t="n">
@@ -21278,7 +21278,7 @@
       <c r="D402" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E402" s="16" t="n">
+      <c r="E402" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F402" s="20" t="n">
@@ -21311,7 +21311,7 @@
       <c r="D403" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E403" s="16" t="n">
+      <c r="E403" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F403" s="20" t="n">
@@ -21344,7 +21344,7 @@
       <c r="D404" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E404" s="16" t="n">
+      <c r="E404" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F404" s="20" t="n">
@@ -21381,7 +21381,7 @@
       <c r="D405" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E405" s="16" t="n">
+      <c r="E405" s="12" t="n">
         <v>1.1386</v>
       </c>
       <c r="F405" s="20" t="n">
@@ -21414,7 +21414,7 @@
       <c r="D406" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E406" s="16" t="n">
+      <c r="E406" s="12" t="n">
         <v>0.4092</v>
       </c>
       <c r="F406" s="20" t="n">
@@ -21447,7 +21447,7 @@
       <c r="D407" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E407" s="16" t="n">
+      <c r="E407" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F407" s="20" t="n">
@@ -21480,7 +21480,7 @@
       <c r="D408" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E408" s="17" t="n">
+      <c r="E408" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F408" s="21" t="n">
@@ -21513,7 +21513,7 @@
       <c r="D409" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="E409" s="16" t="n">
+      <c r="E409" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F409" s="20" t="n">
@@ -21546,7 +21546,7 @@
       <c r="D410" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E410" s="16" t="n">
+      <c r="E410" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F410" s="20" t="n">
@@ -21579,7 +21579,7 @@
       <c r="D411" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E411" s="16" t="n">
+      <c r="E411" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F411" s="20" t="n">
@@ -21612,7 +21612,7 @@
       <c r="D412" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E412" s="16" t="n">
+      <c r="E412" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F412" s="20" t="n">
@@ -21645,7 +21645,7 @@
       <c r="D413" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E413" s="16" t="n">
+      <c r="E413" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F413" s="20" t="n">
@@ -21678,7 +21678,7 @@
       <c r="D414" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E414" s="16" t="n">
+      <c r="E414" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F414" s="20" t="n">
@@ -21711,7 +21711,7 @@
       <c r="D415" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E415" s="16" t="n">
+      <c r="E415" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F415" s="20" t="n">
@@ -21744,7 +21744,7 @@
       <c r="D416" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E416" s="16" t="n">
+      <c r="E416" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F416" s="20" t="n">
@@ -21777,7 +21777,7 @@
       <c r="D417" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E417" s="16" t="n">
+      <c r="E417" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F417" s="20" t="n">
@@ -21810,7 +21810,7 @@
       <c r="D418" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E418" s="16" t="n">
+      <c r="E418" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F418" s="20" t="n">
@@ -21843,7 +21843,7 @@
       <c r="D419" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E419" s="16" t="n">
+      <c r="E419" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F419" s="20" t="n">
@@ -21876,7 +21876,7 @@
       <c r="D420" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E420" s="16" t="n">
+      <c r="E420" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F420" s="20" t="n">
@@ -21909,7 +21909,7 @@
       <c r="D421" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E421" s="16" t="n">
+      <c r="E421" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F421" s="20" t="n">
@@ -21942,7 +21942,7 @@
       <c r="D422" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E422" s="16" t="n">
+      <c r="E422" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F422" s="20" t="n">
@@ -21975,7 +21975,7 @@
       <c r="D423" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E423" s="16" t="n">
+      <c r="E423" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F423" s="20" t="n">
@@ -22008,7 +22008,7 @@
       <c r="D424" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E424" s="16" t="n">
+      <c r="E424" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F424" s="20" t="n">
@@ -22041,7 +22041,7 @@
       <c r="D425" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E425" s="16" t="n">
+      <c r="E425" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F425" s="20" t="n">
@@ -22074,7 +22074,7 @@
       <c r="D426" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E426" s="16" t="n">
+      <c r="E426" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F426" s="20" t="n">
@@ -22107,7 +22107,7 @@
       <c r="D427" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E427" s="16" t="n">
+      <c r="E427" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F427" s="20" t="n">
@@ -22140,7 +22140,7 @@
       <c r="D428" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E428" s="16" t="n">
+      <c r="E428" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F428" s="20" t="n">
@@ -22173,7 +22173,7 @@
       <c r="D429" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E429" s="16" t="n">
+      <c r="E429" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F429" s="20" t="n">
@@ -22210,7 +22210,7 @@
       <c r="D430" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E430" s="17" t="n">
+      <c r="E430" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F430" s="21" t="n">
@@ -22243,7 +22243,7 @@
       <c r="D431" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E431" s="16" t="n">
+      <c r="E431" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F431" s="20" t="n">
@@ -22276,7 +22276,7 @@
       <c r="D432" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E432" s="16" t="n">
+      <c r="E432" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F432" s="20" t="n">
@@ -22309,7 +22309,7 @@
       <c r="D433" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E433" s="16" t="n">
+      <c r="E433" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F433" s="20" t="n">
@@ -22342,7 +22342,7 @@
       <c r="D434" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E434" s="16" t="n">
+      <c r="E434" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F434" s="20" t="n">
@@ -22375,7 +22375,7 @@
       <c r="D435" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E435" s="16" t="n">
+      <c r="E435" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F435" s="20" t="n">
@@ -22408,7 +22408,7 @@
       <c r="D436" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E436" s="16" t="n">
+      <c r="E436" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F436" s="20" t="n">
@@ -22441,7 +22441,7 @@
       <c r="D437" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E437" s="16" t="n">
+      <c r="E437" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F437" s="20" t="n">
@@ -22474,7 +22474,7 @@
       <c r="D438" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E438" s="16" t="n">
+      <c r="E438" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F438" s="20" t="n">
@@ -22507,7 +22507,7 @@
       <c r="D439" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E439" s="16" t="n">
+      <c r="E439" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F439" s="20" t="n">
@@ -22540,7 +22540,7 @@
       <c r="D440" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E440" s="16" t="n">
+      <c r="E440" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F440" s="20" t="n">
@@ -22573,7 +22573,7 @@
       <c r="D441" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E441" s="16" t="n">
+      <c r="E441" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F441" s="20" t="n">
@@ -22606,7 +22606,7 @@
       <c r="D442" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E442" s="16" t="n">
+      <c r="E442" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F442" s="20" t="n">
@@ -22639,7 +22639,7 @@
       <c r="D443" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E443" s="16" t="n">
+      <c r="E443" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F443" s="20" t="n">
@@ -22672,7 +22672,7 @@
       <c r="D444" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E444" s="16" t="n">
+      <c r="E444" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F444" s="20" t="n">
@@ -22705,7 +22705,7 @@
       <c r="D445" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E445" s="16" t="n">
+      <c r="E445" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F445" s="20" t="n">
@@ -22738,7 +22738,7 @@
       <c r="D446" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E446" s="16" t="n">
+      <c r="E446" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F446" s="20" t="n">
@@ -22771,7 +22771,7 @@
       <c r="D447" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E447" s="16" t="n">
+      <c r="E447" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F447" s="20" t="n">
@@ -22804,7 +22804,7 @@
       <c r="D448" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E448" s="16" t="n">
+      <c r="E448" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F448" s="20" t="n">
@@ -22837,7 +22837,7 @@
       <c r="D449" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E449" s="16" t="n">
+      <c r="E449" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F449" s="20" t="n">
@@ -22870,7 +22870,7 @@
       <c r="D450" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E450" s="16" t="n">
+      <c r="E450" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F450" s="20" t="n">
@@ -22903,7 +22903,7 @@
       <c r="D451" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E451" s="16" t="n">
+      <c r="E451" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F451" s="20" t="n">
@@ -22936,7 +22936,7 @@
       <c r="D452" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E452" s="16" t="n">
+      <c r="E452" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F452" s="20" t="n">
@@ -22969,7 +22969,7 @@
       <c r="D453" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E453" s="16" t="n">
+      <c r="E453" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F453" s="20" t="n">
@@ -23002,7 +23002,7 @@
       <c r="D454" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E454" s="16" t="n">
+      <c r="E454" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F454" s="20" t="n">
@@ -23039,7 +23039,7 @@
       <c r="D455" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E455" s="17" t="n">
+      <c r="E455" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F455" s="21" t="n">
@@ -23072,7 +23072,7 @@
       <c r="D456" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E456" s="16" t="n">
+      <c r="E456" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F456" s="20" t="n">
@@ -23105,7 +23105,7 @@
       <c r="D457" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E457" s="16" t="n">
+      <c r="E457" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F457" s="20" t="n">
@@ -23138,7 +23138,7 @@
       <c r="D458" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E458" s="16" t="n">
+      <c r="E458" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F458" s="20" t="n">
@@ -23171,7 +23171,7 @@
       <c r="D459" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E459" s="16" t="n">
+      <c r="E459" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F459" s="20" t="n">
@@ -23204,7 +23204,7 @@
       <c r="D460" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E460" s="16" t="n">
+      <c r="E460" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F460" s="20" t="n">
@@ -23237,7 +23237,7 @@
       <c r="D461" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E461" s="16" t="n">
+      <c r="E461" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F461" s="20" t="n">
@@ -23270,7 +23270,7 @@
       <c r="D462" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E462" s="16" t="n">
+      <c r="E462" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F462" s="20" t="n">
@@ -23303,7 +23303,7 @@
       <c r="D463" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E463" s="16" t="n">
+      <c r="E463" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F463" s="20" t="n">
@@ -23336,7 +23336,7 @@
       <c r="D464" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E464" s="16" t="n">
+      <c r="E464" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F464" s="20" t="n">
@@ -23369,7 +23369,7 @@
       <c r="D465" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E465" s="16" t="n">
+      <c r="E465" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F465" s="20" t="n">
@@ -23402,7 +23402,7 @@
       <c r="D466" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E466" s="16" t="n">
+      <c r="E466" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F466" s="20" t="n">
@@ -23435,7 +23435,7 @@
       <c r="D467" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E467" s="16" t="n">
+      <c r="E467" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F467" s="20" t="n">
@@ -23468,7 +23468,7 @@
       <c r="D468" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E468" s="16" t="n">
+      <c r="E468" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F468" s="20" t="n">
@@ -23501,7 +23501,7 @@
       <c r="D469" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E469" s="16" t="n">
+      <c r="E469" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F469" s="20" t="n">
@@ -23534,7 +23534,7 @@
       <c r="D470" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E470" s="16" t="n">
+      <c r="E470" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F470" s="20" t="n">
@@ -23567,7 +23567,7 @@
       <c r="D471" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E471" s="16" t="n">
+      <c r="E471" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F471" s="20" t="n">
@@ -23600,7 +23600,7 @@
       <c r="D472" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E472" s="16" t="n">
+      <c r="E472" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F472" s="20" t="n">
@@ -23633,7 +23633,7 @@
       <c r="D473" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E473" s="16" t="n">
+      <c r="E473" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F473" s="20" t="n">
@@ -23666,7 +23666,7 @@
       <c r="D474" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E474" s="16" t="n">
+      <c r="E474" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F474" s="20" t="n">
@@ -23699,7 +23699,7 @@
       <c r="D475" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E475" s="16" t="n">
+      <c r="E475" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F475" s="20" t="n">
@@ -23732,7 +23732,7 @@
       <c r="D476" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E476" s="16" t="n">
+      <c r="E476" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F476" s="20" t="n">
@@ -23765,7 +23765,7 @@
       <c r="D477" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E477" s="16" t="n">
+      <c r="E477" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F477" s="20" t="n">
@@ -23798,7 +23798,7 @@
       <c r="D478" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E478" s="16" t="n">
+      <c r="E478" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F478" s="20" t="n">
@@ -23831,7 +23831,7 @@
       <c r="D479" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E479" s="16" t="n">
+      <c r="E479" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F479" s="20" t="n">
@@ -23868,7 +23868,7 @@
       <c r="D480" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E480" s="17" t="n">
+      <c r="E480" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="F480" s="21" t="n">
@@ -23901,7 +23901,7 @@
       <c r="D481" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E481" s="16" t="n">
+      <c r="E481" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F481" s="20" t="n">
@@ -23934,7 +23934,7 @@
       <c r="D482" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E482" s="16" t="n">
+      <c r="E482" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F482" s="20" t="n">
@@ -23967,7 +23967,7 @@
       <c r="D483" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="E483" s="16" t="n">
+      <c r="E483" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F483" s="20" t="n">
@@ -24000,7 +24000,7 @@
       <c r="D484" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E484" s="16" t="n">
+      <c r="E484" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F484" s="20" t="n">
@@ -24033,7 +24033,7 @@
       <c r="D485" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E485" s="16" t="n">
+      <c r="E485" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F485" s="20" t="n">
@@ -24066,7 +24066,7 @@
       <c r="D486" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E486" s="16" t="n">
+      <c r="E486" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F486" s="20" t="n">
@@ -24099,7 +24099,7 @@
       <c r="D487" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E487" s="16" t="n">
+      <c r="E487" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F487" s="20" t="n">
@@ -24132,7 +24132,7 @@
       <c r="D488" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E488" s="16" t="n">
+      <c r="E488" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F488" s="20" t="n">
@@ -24165,7 +24165,7 @@
       <c r="D489" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E489" s="16" t="n">
+      <c r="E489" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F489" s="20" t="n">
@@ -24198,7 +24198,7 @@
       <c r="D490" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E490" s="16" t="n">
+      <c r="E490" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F490" s="20" t="n">
@@ -24231,7 +24231,7 @@
       <c r="D491" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E491" s="16" t="n">
+      <c r="E491" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F491" s="20" t="n">
@@ -24264,7 +24264,7 @@
       <c r="D492" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E492" s="16" t="n">
+      <c r="E492" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F492" s="20" t="n">
@@ -24297,7 +24297,7 @@
       <c r="D493" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E493" s="16" t="n">
+      <c r="E493" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F493" s="20" t="n">
@@ -24330,7 +24330,7 @@
       <c r="D494" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E494" s="16" t="n">
+      <c r="E494" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F494" s="20" t="n">
@@ -24363,7 +24363,7 @@
       <c r="D495" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E495" s="16" t="n">
+      <c r="E495" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F495" s="20" t="n">
@@ -24396,7 +24396,7 @@
       <c r="D496" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E496" s="16" t="n">
+      <c r="E496" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F496" s="20" t="n">
@@ -24429,7 +24429,7 @@
       <c r="D497" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E497" s="16" t="n">
+      <c r="E497" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F497" s="20" t="n">
@@ -24462,7 +24462,7 @@
       <c r="D498" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E498" s="16" t="n">
+      <c r="E498" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F498" s="20" t="n">
@@ -24495,7 +24495,7 @@
       <c r="D499" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E499" s="16" t="n">
+      <c r="E499" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F499" s="20" t="n">
@@ -24528,7 +24528,7 @@
       <c r="D500" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E500" s="16" t="n">
+      <c r="E500" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F500" s="20" t="n">
@@ -24561,7 +24561,7 @@
       <c r="D501" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E501" s="16" t="n">
+      <c r="E501" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F501" s="20" t="n">
@@ -24594,7 +24594,7 @@
       <c r="D502" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E502" s="16" t="n">
+      <c r="E502" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F502" s="20" t="n">
@@ -24627,7 +24627,7 @@
       <c r="D503" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E503" s="16" t="n">
+      <c r="E503" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F503" s="20" t="n">
@@ -24660,7 +24660,7 @@
       <c r="D504" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="E504" s="16" t="n">
+      <c r="E504" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F504" s="20" t="n">

</xml_diff>

<commit_message>
Entregables: regenerar con los barridos del corpus corregido
</commit_message>
<xml_diff>
--- a/docs/Avances_Tesis_Tablas.xlsx
+++ b/docs/Avances_Tesis_Tablas.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Barrido de 25 configuraciones PSO (partículas 2-10 × iteraciones 10-50, Cuadro 1 de Ortega &amp; Espinoza 2025) sobre (r, m), r en [1,25]. El peso converge al piso del rango publicado (m* = 0,30) en las 25 configuraciones, porque Fo decrece de forma estrictamente monótona en m. El radio NO lo fija el PSO: dentro de ese rango Fo prefiere r = 1 (1,7354 frente a 1,7039 en r = 25), de modo que r = 25 es una decisión de diseño tomada sobre las métricas de evaluación, de las cuales cinco lo favorecen (EN, SD, FE, MG, SF) y cuatro prefieren r = 1 (SSIM, PSNR, MI_vis, MI_ir).</t>
+          <t>Barrido de 25 configuraciones PSO (partículas 2-10 × iteraciones 10-50, Cuadro 1 de Ortega &amp; Espinoza 2025) sobre (r, m), r en [1,25]. El peso converge al piso del rango publicado (m* = 0,30) en las 25 configuraciones, porque Fo decrece de forma estrictamente monótona en m. El radio NO lo fija el PSO: dentro de ese rango Fo prefiere r = 1 (1,7350 frente a 1,7057 en r = 25), de modo que r = 25 es una decisión de diseño tomada sobre las métricas de evaluación, de las cuales cinco lo favorecen (EN, SD, FE, MG, SF) y cuatro prefieren r = 1 (SSIM, PSNR, MI_vis, MI_ir).</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Fo = 1.7354</t>
+          <t>Fo = 1.7350</t>
         </is>
       </c>
     </row>
@@ -1865,16 +1865,16 @@
         <v>20</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>1.6988</v>
+        <v>1.699</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -1894,10 +1894,10 @@
         <v>0.3</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -1917,10 +1917,10 @@
         <v>0.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>166</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -1940,10 +1940,10 @@
         <v>0.3</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1963,10 +1963,10 @@
         <v>0.3</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -1986,10 +1986,10 @@
         <v>0.3</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -2009,10 +2009,10 @@
         <v>0.3</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>401</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12">
@@ -2032,10 +2032,10 @@
         <v>0.3</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>86</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13">
@@ -2055,7 +2055,7 @@
         <v>0.3</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G13" s="13" t="n">
         <v>29</v>
@@ -2078,10 +2078,10 @@
         <v>0.3</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G14" s="13" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15">
@@ -2101,10 +2101,10 @@
         <v>0.3</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
@@ -2124,10 +2124,10 @@
         <v>0.3</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -2147,10 +2147,10 @@
         <v>0.3</v>
       </c>
       <c r="F17" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18">
@@ -2170,10 +2170,10 @@
         <v>0.3</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19">
@@ -2193,10 +2193,10 @@
         <v>0.3</v>
       </c>
       <c r="F19" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20">
@@ -2216,10 +2216,10 @@
         <v>0.3</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="G20" s="11" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21">
@@ -2239,7 +2239,7 @@
         <v>0.3</v>
       </c>
       <c r="F21" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>30</v>
@@ -2262,33 +2262,33 @@
         <v>0.3</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="G22" s="11" t="n">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="n">
+      <c r="A23" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B23" s="13" t="n">
+      <c r="B23" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="C23" s="13" t="n">
+      <c r="C23" s="11" t="n">
         <v>320</v>
       </c>
-      <c r="D23" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="14" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F23" s="14" t="n">
-        <v>1.7354</v>
-      </c>
-      <c r="G23" s="13" t="n">
-        <v>136</v>
+      <c r="D23" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="E23" s="12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F23" s="12" t="n">
+        <v>1.7057</v>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>261</v>
       </c>
     </row>
     <row r="24">
@@ -2308,10 +2308,10 @@
         <v>0.3</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>194</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25">
@@ -2331,10 +2331,10 @@
         <v>0.3</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="G25" s="11" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26">
@@ -2354,7 +2354,7 @@
         <v>0.3</v>
       </c>
       <c r="F26" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G26" s="13" t="n">
         <v>40</v>
@@ -2377,10 +2377,10 @@
         <v>0.3</v>
       </c>
       <c r="F27" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="G27" s="13" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28">
@@ -2400,10 +2400,10 @@
         <v>0.3</v>
       </c>
       <c r="F28" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="G28" s="11" t="n">
-        <v>658</v>
+        <v>318</v>
       </c>
     </row>
     <row r="29">
@@ -2423,10 +2423,10 @@
         <v>0.3</v>
       </c>
       <c r="F29" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="G29" s="11" t="n">
-        <v>399</v>
+        <v>409</v>
       </c>
     </row>
     <row r="31">
@@ -2475,19 +2475,19 @@
         </is>
       </c>
       <c r="B33" s="12" t="n">
-        <v>1.6988</v>
+        <v>1.699</v>
       </c>
       <c r="C33" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="D33" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="E33" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="F33" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
     </row>
     <row r="34">
@@ -2497,19 +2497,19 @@
         </is>
       </c>
       <c r="B34" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="C34" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="D34" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="E34" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="F34" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
     </row>
     <row r="35">
@@ -2519,19 +2519,19 @@
         </is>
       </c>
       <c r="B35" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="C35" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="D35" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="E35" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="F35" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
     </row>
     <row r="36">
@@ -2541,19 +2541,19 @@
         </is>
       </c>
       <c r="B36" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="C36" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="D36" s="12" t="n">
-        <v>1.7039</v>
-      </c>
-      <c r="E36" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.7057</v>
+      </c>
+      <c r="E36" s="12" t="n">
+        <v>1.7057</v>
       </c>
       <c r="F36" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
     </row>
     <row r="37">
@@ -2563,19 +2563,19 @@
         </is>
       </c>
       <c r="B37" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="C37" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="D37" s="14" t="n">
-        <v>1.7354</v>
+        <v>1.735</v>
       </c>
       <c r="E37" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.7039</v>
+        <v>1.7057</v>
       </c>
     </row>
     <row r="39">
@@ -7501,7 +7501,7 @@
     <row r="131">
       <c r="A131" s="8" t="inlineStr">
         <is>
-          <t>Triclobs_jeep_in_smoke_R</t>
+          <t>Triclobs_Kaptein_1123</t>
         </is>
       </c>
       <c r="B131" s="9" t="inlineStr">
@@ -7509,32 +7509,32 @@
           <t>Pirámide de Laplace (LP)</t>
         </is>
       </c>
-      <c r="C131" s="18" t="n">
-        <v>6.93067</v>
-      </c>
-      <c r="D131" s="18" t="n">
-        <v>0.14345</v>
-      </c>
-      <c r="E131" s="18" t="n">
-        <v>1.01463</v>
+      <c r="C131" s="19" t="n">
+        <v>7.18866</v>
+      </c>
+      <c r="D131" s="19" t="n">
+        <v>0.20126</v>
+      </c>
+      <c r="E131" s="19" t="n">
+        <v>1.02787</v>
       </c>
       <c r="F131" s="18" t="n">
-        <v>0.03888</v>
-      </c>
-      <c r="G131" s="18" t="n">
-        <v>0.8821</v>
+        <v>0.02132</v>
+      </c>
+      <c r="G131" s="19" t="n">
+        <v>1.18122</v>
       </c>
       <c r="H131" s="19" t="n">
-        <v>1.38236</v>
+        <v>1.98686</v>
       </c>
       <c r="I131" s="18" t="n">
-        <v>22.47202</v>
+        <v>9.284409999999999</v>
       </c>
       <c r="J131" s="18" t="n">
-        <v>0.6109</v>
+        <v>0.7003200000000001</v>
       </c>
       <c r="K131" s="18" t="n">
-        <v>14.06184</v>
+        <v>13.42766</v>
       </c>
     </row>
     <row r="132">
@@ -7545,31 +7545,31 @@
         </is>
       </c>
       <c r="C132" s="18" t="n">
-        <v>7.1874</v>
+        <v>6.714</v>
       </c>
       <c r="D132" s="18" t="n">
-        <v>0.14957</v>
+        <v>0.13217</v>
       </c>
       <c r="E132" s="18" t="n">
-        <v>1.05222</v>
+        <v>0.96</v>
       </c>
       <c r="F132" s="18" t="n">
-        <v>0.04906</v>
+        <v>0.02494</v>
       </c>
       <c r="G132" s="18" t="n">
-        <v>1.32143</v>
+        <v>0.63908</v>
       </c>
       <c r="H132" s="18" t="n">
-        <v>0.93947</v>
+        <v>0.45759</v>
       </c>
       <c r="I132" s="18" t="n">
-        <v>26.71208</v>
+        <v>11.33854</v>
       </c>
       <c r="J132" s="18" t="n">
-        <v>0.59653</v>
+        <v>0.67879</v>
       </c>
       <c r="K132" s="18" t="n">
-        <v>16.34186</v>
+        <v>15.94768</v>
       </c>
     </row>
     <row r="133">
@@ -7580,31 +7580,31 @@
         </is>
       </c>
       <c r="C133" s="18" t="n">
-        <v>7.10092</v>
+        <v>6.71605</v>
       </c>
       <c r="D133" s="18" t="n">
-        <v>0.13585</v>
+        <v>0.1307</v>
       </c>
       <c r="E133" s="18" t="n">
-        <v>1.03956</v>
+        <v>0.9603</v>
       </c>
       <c r="F133" s="18" t="n">
-        <v>0.04219</v>
+        <v>0.0234</v>
       </c>
       <c r="G133" s="18" t="n">
-        <v>1.34031</v>
+        <v>0.84667</v>
       </c>
       <c r="H133" s="18" t="n">
-        <v>1.00889</v>
+        <v>0.70966</v>
       </c>
       <c r="I133" s="18" t="n">
-        <v>23.63965</v>
+        <v>10.76803</v>
       </c>
       <c r="J133" s="18" t="n">
-        <v>0.62621</v>
+        <v>0.70151</v>
       </c>
       <c r="K133" s="18" t="n">
-        <v>16.62357</v>
+        <v>16.2381</v>
       </c>
     </row>
     <row r="134">
@@ -7615,31 +7615,31 @@
         </is>
       </c>
       <c r="C134" s="18" t="n">
-        <v>7.10352</v>
+        <v>6.724</v>
       </c>
       <c r="D134" s="18" t="n">
-        <v>0.13673</v>
+        <v>0.13193</v>
       </c>
       <c r="E134" s="18" t="n">
-        <v>1.03994</v>
+        <v>0.96143</v>
       </c>
       <c r="F134" s="18" t="n">
-        <v>0.04012</v>
-      </c>
-      <c r="G134" s="19" t="n">
-        <v>1.38081</v>
+        <v>0.02094</v>
+      </c>
+      <c r="G134" s="18" t="n">
+        <v>0.8519600000000001</v>
       </c>
       <c r="H134" s="18" t="n">
-        <v>0.99291</v>
+        <v>0.70386</v>
       </c>
       <c r="I134" s="18" t="n">
-        <v>22.59167</v>
+        <v>9.12002</v>
       </c>
       <c r="J134" s="19" t="n">
-        <v>0.6383799999999999</v>
+        <v>0.72489</v>
       </c>
       <c r="K134" s="18" t="n">
-        <v>16.6409</v>
+        <v>16.23278</v>
       </c>
     </row>
     <row r="135">
@@ -7650,31 +7650,31 @@
         </is>
       </c>
       <c r="C135" s="18" t="n">
-        <v>7.06123</v>
+        <v>6.68842</v>
       </c>
       <c r="D135" s="18" t="n">
-        <v>0.13242</v>
+        <v>0.12784</v>
       </c>
       <c r="E135" s="18" t="n">
-        <v>1.03375</v>
+        <v>0.95634</v>
       </c>
       <c r="F135" s="18" t="n">
-        <v>0.0416</v>
+        <v>0.02183</v>
       </c>
       <c r="G135" s="18" t="n">
-        <v>1.30723</v>
+        <v>0.85902</v>
       </c>
       <c r="H135" s="18" t="n">
-        <v>0.98019</v>
+        <v>0.7168600000000001</v>
       </c>
       <c r="I135" s="18" t="n">
-        <v>22.92362</v>
+        <v>9.413040000000001</v>
       </c>
       <c r="J135" s="18" t="n">
-        <v>0.63071</v>
+        <v>0.7144</v>
       </c>
       <c r="K135" s="19" t="n">
-        <v>16.69141</v>
+        <v>16.29629</v>
       </c>
     </row>
     <row r="136">
@@ -7685,31 +7685,31 @@
         </is>
       </c>
       <c r="C136" s="18" t="n">
-        <v>7.3674</v>
+        <v>6.92661</v>
       </c>
       <c r="D136" s="18" t="n">
-        <v>0.16592</v>
+        <v>0.13896</v>
       </c>
       <c r="E136" s="18" t="n">
-        <v>1.07857</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="F136" s="19" t="n">
-        <v>0.08152</v>
+        <v>0.03862</v>
       </c>
       <c r="G136" s="18" t="n">
-        <v>0.8535199999999999</v>
+        <v>0.69873</v>
       </c>
       <c r="H136" s="18" t="n">
-        <v>0.53748</v>
+        <v>0.53608</v>
       </c>
       <c r="I136" s="19" t="n">
-        <v>44.90313</v>
+        <v>15.95473</v>
       </c>
       <c r="J136" s="18" t="n">
-        <v>0.45636</v>
+        <v>0.57725</v>
       </c>
       <c r="K136" s="18" t="n">
-        <v>15.54351</v>
+        <v>15.98544</v>
       </c>
     </row>
     <row r="137">
@@ -7719,38 +7719,38 @@
           <t>PROPUESTA NOVEDOSA (r=25, m=0,30)</t>
         </is>
       </c>
-      <c r="C137" s="19" t="n">
-        <v>7.39259</v>
-      </c>
-      <c r="D137" s="19" t="n">
-        <v>0.17707</v>
-      </c>
-      <c r="E137" s="19" t="n">
-        <v>1.08226</v>
+      <c r="C137" s="18" t="n">
+        <v>6.98109</v>
+      </c>
+      <c r="D137" s="18" t="n">
+        <v>0.15508</v>
+      </c>
+      <c r="E137" s="18" t="n">
+        <v>0.99819</v>
       </c>
       <c r="F137" s="18" t="n">
-        <v>0.05851</v>
+        <v>0.02884</v>
       </c>
       <c r="G137" s="18" t="n">
-        <v>1.25104</v>
+        <v>0.7872400000000001</v>
       </c>
       <c r="H137" s="18" t="n">
-        <v>0.93977</v>
+        <v>0.67077</v>
       </c>
       <c r="I137" s="18" t="n">
-        <v>32.4941</v>
+        <v>12.38207</v>
       </c>
       <c r="J137" s="18" t="n">
-        <v>0.56818</v>
+        <v>0.67193</v>
       </c>
       <c r="K137" s="18" t="n">
-        <v>15.60396</v>
+        <v>15.78024</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
         <is>
-          <t>Triclobs_Kaptein_1123</t>
+          <t>Triclobs_jeep_in_smoke_R</t>
         </is>
       </c>
       <c r="B138" s="9" t="inlineStr">
@@ -7758,32 +7758,32 @@
           <t>Pirámide de Laplace (LP)</t>
         </is>
       </c>
-      <c r="C138" s="19" t="n">
-        <v>7.18866</v>
-      </c>
-      <c r="D138" s="19" t="n">
-        <v>0.20126</v>
-      </c>
-      <c r="E138" s="19" t="n">
-        <v>1.02787</v>
+      <c r="C138" s="18" t="n">
+        <v>6.93067</v>
+      </c>
+      <c r="D138" s="18" t="n">
+        <v>0.14345</v>
+      </c>
+      <c r="E138" s="18" t="n">
+        <v>1.01463</v>
       </c>
       <c r="F138" s="18" t="n">
-        <v>0.02132</v>
-      </c>
-      <c r="G138" s="19" t="n">
-        <v>1.18122</v>
+        <v>0.03888</v>
+      </c>
+      <c r="G138" s="18" t="n">
+        <v>0.8821</v>
       </c>
       <c r="H138" s="19" t="n">
-        <v>1.98686</v>
+        <v>1.38236</v>
       </c>
       <c r="I138" s="18" t="n">
-        <v>9.284409999999999</v>
+        <v>22.47202</v>
       </c>
       <c r="J138" s="18" t="n">
-        <v>0.7003200000000001</v>
+        <v>0.6109</v>
       </c>
       <c r="K138" s="18" t="n">
-        <v>13.42766</v>
+        <v>14.06184</v>
       </c>
     </row>
     <row r="139">
@@ -7794,31 +7794,31 @@
         </is>
       </c>
       <c r="C139" s="18" t="n">
-        <v>6.714</v>
+        <v>7.1874</v>
       </c>
       <c r="D139" s="18" t="n">
-        <v>0.13217</v>
+        <v>0.14957</v>
       </c>
       <c r="E139" s="18" t="n">
-        <v>0.96</v>
+        <v>1.05222</v>
       </c>
       <c r="F139" s="18" t="n">
-        <v>0.02494</v>
+        <v>0.04906</v>
       </c>
       <c r="G139" s="18" t="n">
-        <v>0.63908</v>
+        <v>1.32143</v>
       </c>
       <c r="H139" s="18" t="n">
-        <v>0.45759</v>
+        <v>0.93947</v>
       </c>
       <c r="I139" s="18" t="n">
-        <v>11.33854</v>
+        <v>26.71208</v>
       </c>
       <c r="J139" s="18" t="n">
-        <v>0.67879</v>
+        <v>0.59653</v>
       </c>
       <c r="K139" s="18" t="n">
-        <v>15.94768</v>
+        <v>16.34186</v>
       </c>
     </row>
     <row r="140">
@@ -7829,31 +7829,31 @@
         </is>
       </c>
       <c r="C140" s="18" t="n">
-        <v>6.71605</v>
+        <v>7.10092</v>
       </c>
       <c r="D140" s="18" t="n">
-        <v>0.1307</v>
+        <v>0.13585</v>
       </c>
       <c r="E140" s="18" t="n">
-        <v>0.9603</v>
+        <v>1.03956</v>
       </c>
       <c r="F140" s="18" t="n">
-        <v>0.0234</v>
+        <v>0.04219</v>
       </c>
       <c r="G140" s="18" t="n">
-        <v>0.84667</v>
+        <v>1.34031</v>
       </c>
       <c r="H140" s="18" t="n">
-        <v>0.70966</v>
+        <v>1.00889</v>
       </c>
       <c r="I140" s="18" t="n">
-        <v>10.76803</v>
+        <v>23.63965</v>
       </c>
       <c r="J140" s="18" t="n">
-        <v>0.70151</v>
+        <v>0.62621</v>
       </c>
       <c r="K140" s="18" t="n">
-        <v>16.2381</v>
+        <v>16.62357</v>
       </c>
     </row>
     <row r="141">
@@ -7864,31 +7864,31 @@
         </is>
       </c>
       <c r="C141" s="18" t="n">
-        <v>6.724</v>
+        <v>7.10352</v>
       </c>
       <c r="D141" s="18" t="n">
-        <v>0.13193</v>
+        <v>0.13673</v>
       </c>
       <c r="E141" s="18" t="n">
-        <v>0.96143</v>
+        <v>1.03994</v>
       </c>
       <c r="F141" s="18" t="n">
-        <v>0.02094</v>
-      </c>
-      <c r="G141" s="18" t="n">
-        <v>0.8519600000000001</v>
+        <v>0.04012</v>
+      </c>
+      <c r="G141" s="19" t="n">
+        <v>1.38081</v>
       </c>
       <c r="H141" s="18" t="n">
-        <v>0.70386</v>
+        <v>0.99291</v>
       </c>
       <c r="I141" s="18" t="n">
-        <v>9.12002</v>
+        <v>22.59167</v>
       </c>
       <c r="J141" s="19" t="n">
-        <v>0.72489</v>
+        <v>0.6383799999999999</v>
       </c>
       <c r="K141" s="18" t="n">
-        <v>16.23278</v>
+        <v>16.6409</v>
       </c>
     </row>
     <row r="142">
@@ -7899,31 +7899,31 @@
         </is>
       </c>
       <c r="C142" s="18" t="n">
-        <v>6.68842</v>
+        <v>7.06123</v>
       </c>
       <c r="D142" s="18" t="n">
-        <v>0.12784</v>
+        <v>0.13242</v>
       </c>
       <c r="E142" s="18" t="n">
-        <v>0.95634</v>
+        <v>1.03375</v>
       </c>
       <c r="F142" s="18" t="n">
-        <v>0.02183</v>
+        <v>0.0416</v>
       </c>
       <c r="G142" s="18" t="n">
-        <v>0.85902</v>
+        <v>1.30723</v>
       </c>
       <c r="H142" s="18" t="n">
-        <v>0.7168600000000001</v>
+        <v>0.98019</v>
       </c>
       <c r="I142" s="18" t="n">
-        <v>9.413040000000001</v>
+        <v>22.92362</v>
       </c>
       <c r="J142" s="18" t="n">
-        <v>0.7144</v>
+        <v>0.63071</v>
       </c>
       <c r="K142" s="19" t="n">
-        <v>16.29629</v>
+        <v>16.69141</v>
       </c>
     </row>
     <row r="143">
@@ -7934,31 +7934,31 @@
         </is>
       </c>
       <c r="C143" s="18" t="n">
-        <v>6.92661</v>
+        <v>7.3674</v>
       </c>
       <c r="D143" s="18" t="n">
-        <v>0.13896</v>
+        <v>0.16592</v>
       </c>
       <c r="E143" s="18" t="n">
-        <v>0.9903999999999999</v>
+        <v>1.07857</v>
       </c>
       <c r="F143" s="19" t="n">
-        <v>0.03862</v>
+        <v>0.08152</v>
       </c>
       <c r="G143" s="18" t="n">
-        <v>0.69873</v>
+        <v>0.8535199999999999</v>
       </c>
       <c r="H143" s="18" t="n">
-        <v>0.53608</v>
+        <v>0.53748</v>
       </c>
       <c r="I143" s="19" t="n">
-        <v>15.95473</v>
+        <v>44.90313</v>
       </c>
       <c r="J143" s="18" t="n">
-        <v>0.57725</v>
+        <v>0.45636</v>
       </c>
       <c r="K143" s="18" t="n">
-        <v>15.98544</v>
+        <v>15.54351</v>
       </c>
     </row>
     <row r="144">
@@ -7968,32 +7968,32 @@
           <t>PROPUESTA NOVEDOSA (r=25, m=0,30)</t>
         </is>
       </c>
-      <c r="C144" s="18" t="n">
-        <v>6.98109</v>
-      </c>
-      <c r="D144" s="18" t="n">
-        <v>0.15508</v>
-      </c>
-      <c r="E144" s="18" t="n">
-        <v>0.99819</v>
+      <c r="C144" s="19" t="n">
+        <v>7.39259</v>
+      </c>
+      <c r="D144" s="19" t="n">
+        <v>0.17707</v>
+      </c>
+      <c r="E144" s="19" t="n">
+        <v>1.08226</v>
       </c>
       <c r="F144" s="18" t="n">
-        <v>0.02884</v>
+        <v>0.05851</v>
       </c>
       <c r="G144" s="18" t="n">
-        <v>0.7872400000000001</v>
+        <v>1.25104</v>
       </c>
       <c r="H144" s="18" t="n">
-        <v>0.67077</v>
+        <v>0.93977</v>
       </c>
       <c r="I144" s="18" t="n">
-        <v>12.38207</v>
+        <v>32.4941</v>
       </c>
       <c r="J144" s="18" t="n">
-        <v>0.67193</v>
+        <v>0.56818</v>
       </c>
       <c r="K144" s="18" t="n">
-        <v>15.78024</v>
+        <v>15.60396</v>
       </c>
     </row>
     <row r="146">
@@ -25397,69 +25397,69 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Triclobs_jeep_in_smoke_R</t>
+          <t>Triclobs_Kaptein_1123</t>
         </is>
       </c>
       <c r="B23" s="16" t="n">
-        <v>7.3926</v>
+        <v>6.9811</v>
       </c>
       <c r="C23" s="16" t="n">
-        <v>0.1771</v>
+        <v>0.1551</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>1.0823</v>
+        <v>0.9982</v>
       </c>
       <c r="E23" s="16" t="n">
-        <v>0.0585</v>
+        <v>0.0288</v>
       </c>
       <c r="F23" s="16" t="n">
-        <v>1.251</v>
+        <v>0.7872</v>
       </c>
       <c r="G23" s="16" t="n">
-        <v>0.9398</v>
+        <v>0.6708</v>
       </c>
       <c r="H23" s="16" t="n">
-        <v>32.4941</v>
+        <v>12.3821</v>
       </c>
       <c r="I23" s="16" t="n">
-        <v>0.5682</v>
+        <v>0.6719000000000001</v>
       </c>
       <c r="J23" s="16" t="n">
-        <v>15.604</v>
+        <v>15.7802</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Triclobs_Kaptein_1123</t>
+          <t>Triclobs_jeep_in_smoke_R</t>
         </is>
       </c>
       <c r="B24" s="16" t="n">
-        <v>6.9811</v>
+        <v>7.3926</v>
       </c>
       <c r="C24" s="16" t="n">
-        <v>0.1551</v>
+        <v>0.1771</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>0.9982</v>
+        <v>1.0823</v>
       </c>
       <c r="E24" s="16" t="n">
-        <v>0.0288</v>
+        <v>0.0585</v>
       </c>
       <c r="F24" s="16" t="n">
-        <v>0.7872</v>
+        <v>1.251</v>
       </c>
       <c r="G24" s="16" t="n">
-        <v>0.6708</v>
+        <v>0.9398</v>
       </c>
       <c r="H24" s="16" t="n">
-        <v>12.3821</v>
+        <v>32.4941</v>
       </c>
       <c r="I24" s="16" t="n">
-        <v>0.6719000000000001</v>
+        <v>0.5682</v>
       </c>
       <c r="J24" s="16" t="n">
-        <v>15.7802</v>
+        <v>15.604</v>
       </c>
     </row>
     <row r="25">

</xml_diff>